<commit_message>
Civ Pro attack outline: expand Rule 24(a)(2) intervention row with timeliness
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -1740,22 +1740,22 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Intervention as of right (Rule 24)</t>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Must show: (1) timely; (2) interest in the suit that is at risk; (3) existing parties don't adequately represent it.</t>
+          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>All three are required.</t>
+          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "can intervene because of diversity."</t>
+          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Intervention as of right (Rule 24)</t>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Intervention as of right (Rule 24)</t>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Civ Pro attack outline: clarify forum-defendant removal rule row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -1010,22 +1010,22 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Forum-defendant rule</t>
+          <t>Forum-defendant rule: defendant from the FORUM STATE can't remove on DIVERSITY</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>A defendant sued in his HOME state can't remove ONLY when the basis is diversity.</t>
+          <t>If ANY defendant is a citizen of the state where the suit was filed (the forum state), the case CANNOT be removed when the only basis is DIVERSITY.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Federal-question cases can be removed by a home-state defendant (Marcus, NY v. NY).</t>
+          <t>Ask two questions: (1) Is any defendant from the forum state? (2) Is the only removal basis diversity? Yes to both = NO removal. If there's a FEDERAL QUESTION, a home-state defendant CAN remove (Marcus, NY v. NY).</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "can't remove because he's from the forum state" in a federal-question case.</t>
+          <t>Wrong: "can't remove because he's from the forum state" in a FEDERAL-QUESTION case. Wrong: "can remove on diversity because the parties are diverse" when the defendant is a forum-state citizen.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Forum-defendant rule</t>
+          <t>Forum-defendant rule: defendant from the FORUM STATE can't remove on DIVERSITY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Civ Pro attack outline: add choice-of-law clause row (26A)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$G$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Index'!$A$1:$F$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Everything the defendant INTENTIONALLY did in the forum: living there, contracting there, driving its roads, ads aimed at forum residents, banners meant to attract them.</t>
+          <t>Everything the defendant INTENTIONALLY did in the forum: living there, contracting there, driving its roads, ads aimed at forum residents, banners meant to attract them. A contract clause choosing that state's LAW also counts as evidence (row 26A).</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>The plaintiff's own forum ties can show STATE INTEREST only, never the defendant's contacts. A choice-of-LAW clause can help show interest and purposeful availment.</t>
+          <t>The plaintiff's own forum ties can show STATE INTEREST only, never the defendant's contacts. A choice-of-LAW clause can help show state interest (see row 26A).</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -1513,22 +1513,22 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Forum-selection clauses</t>
+          <t>Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Parties include them to limit exposure to suit everywhere, plan for litigation and pick a convenient forum.</t>
+          <t>Example: "Any litigation about this contract will be brought in the courts of Illinois." Parties include it to (1) limit exposure to being sued everywhere (e.g., a national company worried about general jx); (2) plan for potential lawsuits by defining where suit can be brought; (3) pick a convenient forum. All are valid reasons.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>The clause can't override what the forum's long-arm statute requires.</t>
+          <t>The clause can't override what the forum's long-arm statute requires. Compare row 26A: a choice-of-LAW clause says WHICH LAW applies, not where to sue.</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Choice of FORUM ≠ choice of LAW.</t>
+          <t>Wrong: "these provisions are not enforceable." Choice of FORUM ≠ choice of LAW.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -1538,235 +1538,237 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>26A</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>8. SPECIFIC PJ</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Choice-of-LAW clause: WHICH STATE'S LAW governs, and what it shows for PJ</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Example: "This contract is to be interpreted under the laws of Wisconsin, regardless of the forum." It picks the governing law, NOT the place of suit. But in a PJ challenge it is evidence for two parts of the constitutional test: (1) the chosen state is INTERESTED in the suit; (2) the party PURPOSEFULLY AVAILED itself of that state.</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Party sued in the chosen-law state and challenging PJ? Use the clause as evidence of STATE INTEREST + PURPOSEFUL AVAILMENT (answer: "A and B"). It's evidence, not consent to jurisdiction there; still run the long-arm and the rest of the test.</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "it establishes TRANSIENT jx" (transient = served while physically present). Wrong: "all of the above" when transient is one of the choices. Wrong: treating it as a choice-of-forum clause.</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>21Q26</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>9. NOTICE / SERVICE</t>
         </is>
       </c>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>9. NOTICE / SERVICE</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Notice standard</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Give as much notice as is reasonable given what you know about each defendant; different defendants may get different notice.</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>Known address: serve there. Unknown/pseudonymous: more limited methods.</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Wrong: "publication suffices for both," "no notice to the unknown one," "follow state court rules."</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>21Q16, 20Q1</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
-      <c r="B38" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>10. VENUE</t>
         </is>
       </c>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>10. VENUE</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>§1391 residence venue</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Venue is proper in any district where any defendant resides IF all defendants reside in the same state.</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Defendants in N.D. Ill. and S.D. Ill.: both districts are proper.</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Where the product was designed or parts made doesn't make venue certain.</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>21Q14, 20Q19</t>
-        </is>
-      </c>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>10. VENUE</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>§1391 residence venue</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Venue is proper in any district where any defendant resides IF all defendants reside in the same state.</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Defendants in N.D. Ill. and S.D. Ill.: both districts are proper.</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Where the product was designed or parts made doesn't make venue certain.</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>21Q14, 20Q19</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>10. VENUE</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Dismiss vs. transfer</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>Improper venue: dismissal under Rule 12. Even proper venue: transfer to another district (§1404).</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Venue never sends a case to state court.</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Wrong: "transfer to state court," "dismiss even though venue is proper."</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>21Q6, 20Q8</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
-      <c r="B41" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>11. RULE 12 DEFENSES</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="n">
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>11. RULE 12 DEFENSES</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>What Rule 12(b) can raise</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>No SMJ, no PJ, improper venue, failure to join a Rule 19 party (12(b)(7)).</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>A counterclaim is NOT a Rule 12 defense.</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Defendant can't argue lack of PJ over the plaintiff.</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>21Q15, 20Q54, 20Q56</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-      <c r="B43" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>12. JOINDER</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Intervention as of right (Rule 24(a)(2))</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>21Q7, 20Q4</t>
-        </is>
-      </c>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
@@ -1775,33 +1777,33 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Rule 19 (compulsory joinder)</t>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
+          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
+          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
+          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>21Q8, 20Q20</t>
+          <t>21Q7, 20Q4</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
@@ -1810,33 +1812,33 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Interpleader</t>
+          <t>Rule 19 (compulsory joinder)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
+          <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
+          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Wrong: suing one claimant and impleading the other.</t>
+          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
+          <t>21Q8, 20Q20</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
@@ -1845,108 +1847,112 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
+          <t>Interpleader</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
+          <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
+          <t>Wrong: suing one claimant and impleading the other.</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
+          <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Impleader (Rule 14)</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Limits on joinder</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr"/>
-      <c r="F48" s="3" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>21Q30</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
-      <c r="G49" s="2" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>13. NOT YET COVERED</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Erie (flag: not in Weeks 1-9)</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>Minimum contacts is a PJ test, not Erie.</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>20Q6, 20Q30</t>
-        </is>
-      </c>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
@@ -1955,28 +1961,59 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Forum non conveniens (flag)</t>
+          <t>Erie (flag: not in Weeks 1-9)</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
       <c r="F51" s="5" t="inlineStr">
         <is>
+          <t>Minimum contacts is a PJ test, not Erie.</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>20Q6, 20Q30</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>13. NOT YET COVERED</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Forum non conveniens (flag)</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
           <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>20Q36</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G51"/>
+  <autoFilter ref="A1:G52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2776,7 +2813,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Forum-selection clauses</t>
+          <t>Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2838,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26A, 25, 23</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>State interest</t>
+          <t>Choice-of-LAW clause: WHICH STATE'S LAW governs, and what it shows for PJ; State interest; Purposeful availment</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4373,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Two-step test; Forum-selection clauses</t>
+          <t>Two-step test; Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Civ Pro attack outline: drop # column; index points to real Excel rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$G$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Index'!$A$1:$F$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,1060 +478,968 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Topic</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Topic</t>
+          <t>RULE</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>RULE</t>
+          <t>Test / how to apply</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Test / how to apply</t>
+          <t>Traps (wrong answers the finals used)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Traps (wrong answers the finals used)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>Final Qs</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Sources of SMJ</t>
+        </is>
+      </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Sources of SMJ</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
           <t>Federal SMJ comes from the Constitution (Art. III) and federal statutes (§1331 FQ, §1332 diversity).</t>
         </is>
       </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Two original bases: FEDERAL QUESTION or DIVERSITY. Supplemental only adds claims once a case is properly in.</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Two original bases: FEDERAL QUESTION or DIVERSITY. Supplemental only adds claims once a case is properly in.</t>
+          <t>State long-arm statutes are irrelevant to SMJ (that's PJ).</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>State long-arm statutes are irrelevant to SMJ (that's PJ).</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
           <t>21Q1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Federal question: well-pleaded complaint</t>
+        </is>
+      </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Federal question: well-pleaded complaint</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
           <t>The federal issue must appear in the PLAINTIFF'S COMPLAINT (Mottley).</t>
         </is>
       </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Look only at the complaint's own claim. An anticipated federal DEFENSE doesn't count.</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Look only at the complaint's own claim. An anticipated federal DEFENSE doesn't count.</t>
+          <t>Wrong: "yes if defendant actually raises the federal defense" / "if the case ends up focusing on federal law."</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "yes if defendant actually raises the federal defense" / "if the case ends up focusing on federal law."</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
           <t>21Q5, 20Q12</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Federal question: no amount, no citizenship</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Federal question: no amount, no citizenship</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
           <t>Federal question has NO amount-in-controversy minimum and doesn't care about citizenship.</t>
         </is>
       </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Foreign plaintiff suing on federal law: FQ jurisdiction exists.</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Foreign plaintiff suing on federal law: FQ jurisdiction exists.</t>
+          <t>Wrong: $75,000 / $75,000.01 / $75,001 (those are diversity). Wrong: "a foreign citizen can't sue in federal court."</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Wrong: $75,000 / $75,000.01 / $75,001 (those are diversity). Wrong: "a foreign citizen can't sue in federal court."</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
           <t>21Q24, 20Q18, 20Q51</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Diversity: complete diversity</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Diversity: complete diversity</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
           <t>No plaintiff may share citizenship with ANY defendant, plus amount in controversy &gt; $75,000.</t>
         </is>
       </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Check every P against every D. One overlap kills it.</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Check every P against every D. One overlap kills it.</t>
+          <t>IL+NE plaintiffs v. NE defendants = no diversity. Same-state P and D (Tam v. Ollie) = no diversity even if the co-plaintiff (Kes) is diverse.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>IL+NE plaintiffs v. NE defendants = no diversity. Same-state P and D (Tam v. Ollie) = no diversity even if the co-plaintiff (Kes) is diverse.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
           <t>20Q14, 21Q10, 21Q60</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Diversity: aliens</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Diversity: aliens</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
           <t>There must be a U.S. citizen on at least one side of the v. U.S. citizen v. foreign citizen is diverse.</t>
         </is>
       </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>IL plaintiff v. Canadian defendants = diverse. IL plaintiff v. permanent resident living in Texas = diverse (per 2021 key).</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>IL plaintiff v. Canadian defendants = diverse. IL plaintiff v. permanent resident living in Texas = diverse (per 2021 key).</t>
+          <t>Wrong: "no diversity because the foreign defendant isn't a citizen of any state." Wrong: mixing in PJ ("no PJ over a non-U.S. citizen").</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "no diversity because the foreign defendant isn't a citizen of any state." Wrong: mixing in PJ ("no PJ over a non-U.S. citizen").</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
           <t>20Q35, 21Q10</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>1. SUBJECT MATTER JX</t>
         </is>
       </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Corporations: citizenship vs. general PJ</t>
+        </is>
+      </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Corporations: citizenship vs. general PJ</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
           <t>DIVERSITY: a corporation is a citizen only of its state of incorporation and its principal place of business ("nerve center"), so two at most. GENERAL PJ: anywhere it has continuous and systematic contacts so it is essentially at home.</t>
         </is>
       </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Citizenship is narrow by design; it can't be everywhere the corporation does business.</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Citizenship is narrow by design; it can't be everywhere the corporation does business.</t>
+          <t>Don't swap the two tests. Wrong: "citizen wherever it has continuous and systematic contacts."</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Don't swap the two tests. Wrong: "citizen wherever it has continuous and systematic contacts."</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
           <t>21Q20, 20Q17</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2. DOMICILE</t>
         </is>
       </c>
+      <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>2. DOMICILE</t>
         </is>
       </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Domicile test</t>
+        </is>
+      </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Domicile test</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
           <t>Domicile = physical presence + intent to remain. The old domicile continues until a new one is acquired. Domicile is a legal conclusion, not a fact.</t>
         </is>
       </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>College students usually keep their home domicile (Petia, Duncan): presence without intent to remain doesn't change it.</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>College students usually keep their home domicile (Petia, Duncan): presence without intent to remain doesn't change it.</t>
+          <t>Wrong: "domicile is where they've lived 4 years" / "two domiciles" / "no domicile" / "most recent place (London)."</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "domicile is where they've lived 4 years" / "two domiciles" / "no domicile" / "most recent place (London)."</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
           <t>20Q7, 21Q19, 20Q41</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>2. DOMICILE</t>
         </is>
       </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Why domicile matters</t>
+        </is>
+      </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Why domicile matters</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
           <t>(1) Diversity citizenship of individuals. (2) General PJ over individuals (sued at home for conduct elsewhere).</t>
         </is>
       </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>A plaintiff is NOT limited to suing where she is domiciled.</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>A plaintiff is NOT limited to suing where she is domiciled.</t>
+          <t>Wrong: "it matters for where he is allowed to sue." Right answers pair diversity + general PJ.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "it matters for where he is allowed to sue." Right answers pair diversity + general PJ.</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
           <t>21Q18, 20Q59</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>3. SUPPLEMENTAL JX</t>
         </is>
       </c>
+      <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>3. SUPPLEMENTAL JX</t>
         </is>
       </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>§1367(a): same case or controversy</t>
+        </is>
+      </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>§1367(a): same case or controversy</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
           <t>A joined claim needs supplemental jx if it lacks its own basis: it must arise from the same set of facts as the anchor claim.</t>
         </is>
       </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Supplemental jx only matters when a JOINDER happens (counterclaim, impleader, added claim/party).</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Supplemental jx only matters when a JOINDER happens (counterclaim, impleader, added claim/party).</t>
+          <t>Wrong: "SMJ because the original claim is federal" without asking whether the new claim is related.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "SMJ because the original claim is federal" without asking whether the new claim is related.</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
           <t>21Q28, 21Q29, 20Q33, 20Q47, 20Q58</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>3. SUPPLEMENTAL JX</t>
         </is>
       </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>§1367(b): diversity-only limit</t>
+        </is>
+      </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>§1367(b): diversity-only limit</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
           <t>In a case resting ONLY on diversity, a PLAINTIFF can't use supplemental jx for claims against a non-diverse party joined under Rule 14/19/20/24.</t>
         </is>
       </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>A DEFENDANT'S impleader claim against a non-diverse third party can still be supplemental. With a federal-question anchor, (b) doesn't apply. A plaintiff's claim against a diverse third party works if it independently meets diversity OR arises from the original claim.</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>A DEFENDANT'S impleader claim against a non-diverse third party can still be supplemental. With a federal-question anchor, (b) doesn't apply. A plaintiff's claim against a diverse third party works if it independently meets diversity OR arises from the original claim.</t>
+          <t>Artis (LA) v. Arei (LA, impleaded) = barred. 30R v. MetroFord (both MI, impleader) = may be supplemental.</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Artis (LA) v. Arei (LA, impleaded) = barred. 30R v. MetroFord (both MI, impleader) = may be supplemental.</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
           <t>20Q37, 20Q39, 20Q58, 21Q29</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>3. SUPPLEMENTAL JX</t>
         </is>
       </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Counterclaims and SMJ</t>
+        </is>
+      </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Counterclaims and SMJ</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
           <t>COMPULSORY counterclaim (same transaction): supplemental jx always. PERMISSIVE: may have supplemental jx, or needs its own basis. A compulsory counterclaim not asserted is barred later.</t>
         </is>
       </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>A counterclaim raising its own federal question has SMJ regardless of the parties' citizenship.</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>A counterclaim raising its own federal question has SMJ regardless of the parties' citizenship.</t>
+          <t>Wrong: "same-state P and D destroys SMJ over a federal counterclaim." Wrong: "unasserted compulsory counterclaim can be brought later if diversity exists."</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "same-state P and D destroys SMJ over a federal counterclaim." Wrong: "unasserted compulsory counterclaim can be brought later if diversity exists."</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
           <t>20Q57, 20Q16, 21Q28</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>4. REMOVAL</t>
         </is>
       </c>
+      <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>4. REMOVAL</t>
         </is>
       </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Who and what basis</t>
+        </is>
+      </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Who and what basis</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
           <t>Only the DEFENDANT removes, and must show an original basis (federal question or diversity) on the ORIGINAL complaint.</t>
         </is>
       </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Supplemental jx can't support removal: at removal we look only at the original case, with nothing added.</t>
+        </is>
+      </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Supplemental jx can't support removal: at removal we look only at the original case, with nothing added.</t>
+          <t>Wrong: "plaintiff can remove because he filed." Wrong: "FQ removal requires the amount."</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "plaintiff can remove because he filed." Wrong: "FQ removal requires the amount."</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
           <t>21Q2, 21Q27, 20Q2</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>4. REMOVAL</t>
         </is>
       </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Forum-defendant rule: defendant from the FORUM STATE can't remove on DIVERSITY</t>
+        </is>
+      </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Forum-defendant rule: defendant from the FORUM STATE can't remove on DIVERSITY</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
           <t>If ANY defendant is a citizen of the state where the suit was filed (the forum state), the case CANNOT be removed when the only basis is DIVERSITY.</t>
         </is>
       </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Ask two questions: (1) Is any defendant from the forum state? (2) Is the only removal basis diversity? Yes to both = NO removal. If there's a FEDERAL QUESTION, a home-state defendant CAN remove (Marcus, NY v. NY).</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Ask two questions: (1) Is any defendant from the forum state? (2) Is the only removal basis diversity? Yes to both = NO removal. If there's a FEDERAL QUESTION, a home-state defendant CAN remove (Marcus, NY v. NY).</t>
+          <t>Wrong: "can't remove because he's from the forum state" in a FEDERAL-QUESTION case. Wrong: "can remove on diversity because the parties are diverse" when the defendant is a forum-state citizen.</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "can't remove because he's from the forum state" in a FEDERAL-QUESTION case. Wrong: "can remove on diversity because the parties are diverse" when the defendant is a forum-state citizen.</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
           <t>20Q15, 21Q2</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>4. REMOVAL</t>
         </is>
       </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Where it goes / routes</t>
+        </is>
+      </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Where it goes / routes</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
           <t>Removal goes to the federal district court for the district embracing the state court (§1446/§1441(a)). Routes from state to federal: (1) removal to the federal trial court; (2) U.S. Supreme Court review after the state's highest court.</t>
         </is>
       </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>No appeal from a state trial court to a federal court of appeals.</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>No appeal from a state trial court to a federal court of appeals.</t>
+          <t>Wrong: "nearest federal court in the defendant's state."</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "nearest federal court in the defendant's state."</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
           <t>21Q3, 21Q54</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>5. PERSONAL JX: FRAMEWORK</t>
         </is>
       </c>
+      <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>5. PERSONAL JX: FRAMEWORK</t>
         </is>
       </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Two-step test</t>
+        </is>
+      </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Two-step test</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
           <t>Plaintiff must show (1) the FORUM state's long-arm statute is met AND (2) exercising jx is constitutional (due process).</t>
         </is>
       </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Use the long-arm of the forum, not the plaintiff's or defendant's home state. If the long-arm isn't met, stop: no PJ even if the Constitution would allow it.</t>
+        </is>
+      </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Use the long-arm of the forum, not the plaintiff's or defendant's home state. If the long-arm isn't met, stop: no PJ even if the Constitution would allow it.</t>
+          <t>A statute of limitations is NOT a long-arm statute. A choice-of-forum clause can't override the forum's long-arm.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>A statute of limitations is NOT a long-arm statute. A choice-of-forum clause can't override the forum's long-arm.</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
           <t>20Q48, 20Q23, 20Q32</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>5. PERSONAL JX: FRAMEWORK</t>
         </is>
       </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Federal courts borrow the long-arm</t>
+        </is>
+      </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Federal courts borrow the long-arm</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
           <t>Federal courts have no long-arm of their own; they borrow the long-arm of the state where they sit (FRCP 4). The PJ analysis is the same in a state's state and federal courts.</t>
         </is>
       </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>A federal court in Illinois uses the Illinois long-arm plus the constitutional test.</t>
+        </is>
+      </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>A federal court in Illinois uses the Illinois long-arm plus the constitutional test.</t>
+          <t>Wrong: "federal court long-arm statute," "plaintiff's/defendant's home long-arm," "different standards in state vs. federal court."</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "federal court long-arm statute," "plaintiff's/defendant's home long-arm," "different standards in state vs. federal court."</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
           <t>21Q4, 20Q3, 21Q17, 20Q50</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>5. PERSONAL JX: FRAMEWORK</t>
         </is>
       </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Whose rights; modern focus</t>
+        </is>
+      </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Whose rights; modern focus</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
           <t>The constitutional analysis protects the DEFENDANT'S due process rights. The modern test focuses on the defendant's connections and fairness.</t>
         </is>
       </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff consents to PJ by filing, so a defendant can't challenge PJ "over the plaintiff."</t>
+        </is>
+      </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Plaintiff consents to PJ by filing, so a defendant can't challenge PJ "over the plaintiff."</t>
+          <t>Wrong: plaintiff's due process, state sovereignty, full faith and credit.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Wrong: plaintiff's due process, state sovereignty, full faith and credit.</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
           <t>20Q38, 21Q59, 20Q34, 20Q56</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>6. PENNOYER / TRANSIENT</t>
         </is>
       </c>
+      <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>6. PENNOYER / TRANSIENT</t>
         </is>
       </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Pennoyer (old rule)</t>
+        </is>
+      </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Pennoyer (old rule)</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
           <t>PJ if the defendant was physically present in the state when served OR his property in the state was seized BEFORE the suit began.</t>
         </is>
       </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>What matters: where the defendant was when served.</t>
+        </is>
+      </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>What matters: where the defendant was when served.</t>
+          <t>Wrong: property seized AFTER suit began; "knew/foreseeable he could be sued there"; minimum contacts (that's modern).</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Wrong: property seized AFTER suit began; "knew/foreseeable he could be sued there"; minimum contacts (that's modern).</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
           <t>21Q9, 20Q5, 21Q55</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>6. PENNOYER / TRANSIENT</t>
         </is>
       </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Transient (tag) jurisdiction survives</t>
+        </is>
+      </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Transient (tag) jurisdiction survives</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
           <t>Served while physically present in the forum = PJ. No other contacts needed.</t>
         </is>
       </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Wanesa served while briefly stopping in Ohio; Antoni served on vacation in California: PJ.</t>
+        </is>
+      </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Wanesa served while briefly stopping in Ohio; Antoni served on vacation in California: PJ.</t>
+          <t>Wrong: "Pennoyer's rule disappeared with minimum contacts" / "depends on other contacts."</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "Pennoyer's rule disappeared with minimum contacts" / "depends on other contacts."</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
           <t>21Q11, 20Q9, 21Q37, 20Q53</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>7. GENERAL PJ</t>
         </is>
       </c>
+      <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>7. GENERAL PJ</t>
         </is>
       </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Test and where</t>
+        </is>
+      </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Test and where</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
           <t>Defendant is ESSENTIALLY AT HOME (continuous and systematic contacts). Applies to individuals (domicile) and corporations.</t>
         </is>
       </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Corporation: safe forums are its state of incorporation and headquarters/main facility state (BT: FL and GA; Flags: VT and GA).</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Corporation: safe forums are its state of incorporation and headquarters/main facility state (BT: FL and GA; Flags: VT and GA).</t>
+          <t>Wrong: "minimum contacts," "purposeful availment," "one contract," "no general jx over individuals/internet companies."</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "minimum contacts," "purposeful availment," "one contract," "no general jx over individuals/internet companies."</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
           <t>21Q38, 21Q58, 20Q13, 21Q40</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>7. GENERAL PJ</t>
         </is>
       </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>General vs. specific</t>
+        </is>
+      </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>General vs. specific</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
           <t>General jx is a HIGHER standard than purposeful availment (purposeful availment over a range of areas). Both general and specific jx can exist in multiple places.</t>
         </is>
       </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>If purposeful availment fails, general jx fails too.</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>If purposeful availment fails, general jx fails too.</t>
+          <t>Wrong: "only one place for general jx" / "if no specific, there must be general."</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "only one place for general jx" / "if no specific, there must be general."</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
           <t>21Q39, 20Q49, 21Q51</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Elements</t>
+        </is>
+      </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Elements</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
           <t>(1) Purposeful availment; (2) suit arises out of/relates to the defendant's forum contacts; (3) state interest; (4) reasonableness.</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>All four must be proven when the defendant isn't domiciled in the forum.</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>20Q60, 20Q22</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Purposeful availment</t>
+        </is>
+      </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Purposeful availment</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Everything the defendant INTENTIONALLY did in the forum: living there, contracting there, driving its roads, ads aimed at forum residents, banners meant to attract them. A contract clause choosing that state's LAW also counts as evidence (row 26A).</t>
+          <t>Everything the defendant INTENTIONALLY did in the forum: living there, contracting there, driving its roads, ads aimed at forum residents, banners meant to attract them. A contract clause choosing that state's LAW also counts as evidence (see the Choice-of-LAW clause row).</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Purposeful availment doesn't screen related vs. unrelated contacts (that's "arises out of").</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Purposeful availment doesn't screen related vs. unrelated contacts (that's "arises out of").</t>
+          <t>Wrong: "reasonably foreseeable the product would end up there" alone. Minimum contacts is much less than general jx.</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "reasonably foreseeable the product would end up there" alone. Minimum contacts is much less than general jx.</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
           <t>20Q55, 21Q52, 20Q25, 20Q26, 20Q24</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Arises out of / relates to</t>
+        </is>
+      </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Arises out of / relates to</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
           <t>The suit springs from or relates to the DEFENDANT'S contacts with the forum.</t>
         </is>
       </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Not the plaintiff's contacts.</t>
+        </is>
+      </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Not the plaintiff's contacts.</t>
+          <t>Wrong: "suit sprang from the plaintiff's contacts," "continuous contacts" (general), "a long-arm allows it."</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "suit sprang from the plaintiff's contacts," "continuous contacts" (general), "a long-arm allows it."</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
           <t>21Q36</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>State interest</t>
+        </is>
+      </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>State interest</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
           <t>A state is interested if the plaintiff is from there or the tort occurred there. Being the forum alone isn't enough.</t>
         </is>
       </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>The plaintiff's own forum ties can show STATE INTEREST only, never the defendant's contacts. A choice-of-LAW clause can help show state interest (see the Choice-of-LAW clause row).</t>
+        </is>
+      </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>The plaintiff's own forum ties can show STATE INTEREST only, never the defendant's contacts. A choice-of-LAW clause can help show state interest (see row 26A).</t>
+          <t>Wrong: "the forum state is always interested."</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "the forum state is always interested."</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
           <t>21Q53, 20Q27, 21Q43, 21Q26</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
+        </is>
+      </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
           <t>Example: "Any litigation about this contract will be brought in the courts of Illinois." Parties include it to (1) limit exposure to being sued everywhere (e.g., a national company worried about general jx); (2) plan for potential lawsuits by defining where suit can be brought; (3) pick a convenient forum. All are valid reasons.</t>
         </is>
       </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>The clause can't override what the forum's long-arm statute requires. Compare the next row: a choice-of-LAW clause says WHICH LAW applies, not where to sue.</t>
+        </is>
+      </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>The clause can't override what the forum's long-arm statute requires. Compare row 26A: a choice-of-LAW clause says WHICH LAW applies, not where to sue.</t>
+          <t>Wrong: "these provisions are not enforceable." Choice of FORUM ≠ choice of LAW.</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Wrong: "these provisions are not enforceable." Choice of FORUM ≠ choice of LAW.</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>21Q25, 20Q32</t>
         </is>
@@ -1540,480 +1448,437 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>26A</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Choice-of-LAW clause: WHICH STATE'S LAW governs, and what it shows for PJ</t>
+        </is>
+      </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Choice-of-LAW clause: WHICH STATE'S LAW governs, and what it shows for PJ</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
           <t>Example: "This contract is to be interpreted under the laws of Wisconsin, regardless of the forum." It picks the governing law, NOT the place of suit. But in a PJ challenge it is evidence for two parts of the constitutional test: (1) the chosen state is INTERESTED in the suit; (2) the party PURPOSEFULLY AVAILED itself of that state.</t>
         </is>
       </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Party sued in the chosen-law state and challenging PJ? Use the clause as evidence of STATE INTEREST + PURPOSEFUL AVAILMENT (answer: "A and B"). It's evidence, not consent to jurisdiction there; still run the long-arm and the rest of the test.</t>
+        </is>
+      </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Party sued in the chosen-law state and challenging PJ? Use the clause as evidence of STATE INTEREST + PURPOSEFUL AVAILMENT (answer: "A and B"). It's evidence, not consent to jurisdiction there; still run the long-arm and the rest of the test.</t>
+          <t>Wrong: "it establishes TRANSIENT jx" (transient = served while physically present). Wrong: "all of the above" when transient is one of the choices. Wrong: treating it as a choice-of-forum clause.</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "it establishes TRANSIENT jx" (transient = served while physically present). Wrong: "all of the above" when transient is one of the choices. Wrong: treating it as a choice-of-forum clause.</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
           <t>21Q26</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>9. NOTICE / SERVICE</t>
         </is>
       </c>
+      <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="n"/>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>9. NOTICE / SERVICE</t>
         </is>
       </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Notice standard</t>
+        </is>
+      </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Notice standard</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
           <t>Give as much notice as is reasonable given what you know about each defendant; different defendants may get different notice.</t>
         </is>
       </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Known address: serve there. Unknown/pseudonymous: more limited methods.</t>
+        </is>
+      </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Known address: serve there. Unknown/pseudonymous: more limited methods.</t>
+          <t>Wrong: "publication suffices for both," "no notice to the unknown one," "follow state court rules."</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "publication suffices for both," "no notice to the unknown one," "follow state court rules."</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
           <t>21Q16, 20Q1</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>10. VENUE</t>
         </is>
       </c>
+      <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>10. VENUE</t>
         </is>
       </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>§1391 residence venue</t>
+        </is>
+      </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>§1391 residence venue</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
           <t>Venue is proper in any district where any defendant resides IF all defendants reside in the same state.</t>
         </is>
       </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Defendants in N.D. Ill. and S.D. Ill.: both districts are proper.</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Defendants in N.D. Ill. and S.D. Ill.: both districts are proper.</t>
+          <t>Where the product was designed or parts made doesn't make venue certain.</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Where the product was designed or parts made doesn't make venue certain.</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
           <t>21Q14, 20Q19</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>10. VENUE</t>
         </is>
       </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Dismiss vs. transfer</t>
+        </is>
+      </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Dismiss vs. transfer</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
           <t>Improper venue: dismissal under Rule 12. Even proper venue: transfer to another district (§1404).</t>
         </is>
       </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Venue never sends a case to state court.</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Venue never sends a case to state court.</t>
+          <t>Wrong: "transfer to state court," "dismiss even though venue is proper."</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "transfer to state court," "dismiss even though venue is proper."</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
           <t>21Q6, 20Q8</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>11. RULE 12 DEFENSES</t>
         </is>
       </c>
+      <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>11. RULE 12 DEFENSES</t>
         </is>
       </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>What Rule 12(b) can raise</t>
+        </is>
+      </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>What Rule 12(b) can raise</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
           <t>No SMJ, no PJ, improper venue, failure to join a Rule 19 party (12(b)(7)).</t>
         </is>
       </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>A counterclaim is NOT a Rule 12 defense.</t>
+        </is>
+      </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>A counterclaim is NOT a Rule 12 defense.</t>
+          <t>Defendant can't argue lack of PJ over the plaintiff.</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Defendant can't argue lack of PJ over the plaintiff.</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
           <t>21Q15, 20Q54, 20Q56</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
+      <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
+        </is>
+      </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Intervention as of right (Rule 24(a)(2))</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
           <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
         </is>
       </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
+        </is>
+      </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
+          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
           <t>21Q7, 20Q4</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Rule 19 (compulsory joinder)</t>
+        </is>
+      </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Rule 19 (compulsory joinder)</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
           <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
         </is>
       </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
+        </is>
+      </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
+          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
           <t>21Q8, 20Q20</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Interpleader</t>
+        </is>
+      </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Interpleader</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
           <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
         </is>
       </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
+        </is>
+      </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
+          <t>Wrong: suing one claimant and impleading the other.</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Wrong: suing one claimant and impleading the other.</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
           <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Impleader (Rule 14)</t>
+        </is>
+      </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
           <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
         </is>
       </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
           <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Limits on joinder</t>
+        </is>
+      </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Limits on joinder</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
           <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
+        </is>
+      </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
           <t>21Q30</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
+      <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="n"/>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
-      <c r="G50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Erie (flag: not in Weeks 1-9)</t>
+        </is>
+      </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Erie (flag: not in Weeks 1-9)</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
           <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Minimum contacts is a PJ test, not Erie.</t>
+        </is>
+      </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Minimum contacts is a PJ test, not Erie.</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
           <t>20Q6, 20Q30</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Forum non conveniens (flag)</t>
+        </is>
+      </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Forum non conveniens (flag)</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
           <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
+        </is>
+      </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
           <t>20Q36</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G52"/>
+  <autoFilter ref="A1:F52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2058,7 +1923,7 @@
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>Outline row #</t>
+          <t>Attack Outline Excel row</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
@@ -2088,7 +1953,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -2118,7 +1983,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -2148,7 +2013,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -2178,7 +2043,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -2208,7 +2073,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -2238,7 +2103,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>41</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -2268,7 +2133,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -2298,7 +2163,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>46</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -2328,7 +2193,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -2358,7 +2223,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>4, 5</t>
+          <t>6, 7</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -2388,7 +2253,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -2418,7 +2283,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2448,7 +2313,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2478,7 +2343,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2508,7 +2373,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>43</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2538,7 +2403,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2568,7 +2433,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -2598,7 +2463,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2628,7 +2493,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2658,7 +2523,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2688,7 +2553,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2718,7 +2583,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2748,7 +2613,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2778,7 +2643,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2808,7 +2673,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2838,7 +2703,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>26A, 25, 23</t>
+          <t>36, 34, 32</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2868,7 +2733,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2898,7 +2763,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>9, 11</t>
+          <t>13, 15</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -2928,7 +2793,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>9, 10</t>
+          <t>13, 14</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2958,7 +2823,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -2988,7 +2853,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -3018,7 +2883,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -3048,7 +2913,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -3078,7 +2943,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -3108,7 +2973,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -3138,7 +3003,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -3168,7 +3033,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -3198,7 +3063,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>34</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -3228,7 +3093,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -3258,7 +3123,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3288,7 +3153,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -3318,7 +3183,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -3348,7 +3213,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -3378,7 +3243,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -3408,7 +3273,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -3438,7 +3303,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -3468,7 +3333,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -3498,7 +3363,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -3528,7 +3393,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -3558,7 +3423,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -3588,7 +3453,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>51</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -3618,7 +3483,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -3648,7 +3513,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>41</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -3678,7 +3543,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -3708,7 +3573,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -3738,7 +3603,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -3768,7 +3633,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -3798,7 +3663,7 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -3828,7 +3693,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>4, 5</t>
+          <t>6, 7</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -3858,7 +3723,7 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3888,7 +3753,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -3918,7 +3783,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -3948,7 +3813,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -3978,7 +3843,7 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -4008,7 +3873,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>46</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -4038,7 +3903,7 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -4068,7 +3933,7 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
@@ -4098,7 +3963,7 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -4128,7 +3993,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -4158,7 +4023,7 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -4188,7 +4053,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -4218,7 +4083,7 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>34</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -4248,7 +4113,7 @@
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -4278,7 +4143,7 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
@@ -4308,7 +4173,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>51</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -4338,7 +4203,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -4368,7 +4233,7 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>15, 26</t>
+          <t>21, 35</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -4398,7 +4263,7 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -4428,7 +4293,7 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
@@ -4458,7 +4323,7 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -4488,7 +4353,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
@@ -4518,7 +4383,7 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
@@ -4548,7 +4413,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -4578,7 +4443,7 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
@@ -4608,7 +4473,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -4638,7 +4503,7 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -4668,7 +4533,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -4698,7 +4563,7 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>7, 4</t>
+          <t>10, 6</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -4728,7 +4593,7 @@
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>4, 5</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -4758,7 +4623,7 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -4788,7 +4653,7 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -4818,7 +4683,7 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -4848,7 +4713,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -4878,7 +4743,7 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
@@ -4908,7 +4773,7 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
@@ -4938,7 +4803,7 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
@@ -4968,7 +4833,7 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>15, 22</t>
+          <t>21, 31</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -4998,7 +4863,7 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
@@ -5028,7 +4893,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>43</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
@@ -5058,7 +4923,7 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -5088,7 +4953,7 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>17, 30</t>
+          <t>23, 43</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
@@ -5118,7 +4983,7 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -5148,7 +5013,7 @@
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
@@ -5178,7 +5043,7 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
@@ -5208,7 +5073,7 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Civ Pro attack outline: add Rule 13 counterclaim row; fix permissive counterclaim SMJ rule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Index'!$A$1:$F$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -890,17 +890,17 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>COMPULSORY counterclaim (same transaction): supplemental jx always. PERMISSIVE: may have supplemental jx, or needs its own basis. A compulsory counterclaim not asserted is barred later.</t>
+          <t>COMPULSORY counterclaim (same transaction/occurrence as the plaintiff's claim): supplemental jx ALWAYS. PERMISSIVE counterclaim (unrelated): NO supplemental jx; it needs its OWN basis (federal question or diversity).</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>A counterclaim raising its own federal question has SMJ regardless of the parties' citizenship.</t>
+          <t>Ask: does the counterclaim arise out of the original claim? Yes = compulsory = supplemental jx. No = permissive = check FQ/diversity on its own. A counterclaim raising its own federal question has SMJ regardless of the parties' citizenship.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "same-state P and D destroys SMJ over a federal counterclaim." Wrong: "unasserted compulsory counterclaim can be brought later if diversity exists."</t>
+          <t>Wrong: "if permissive, there MAY be supplemental jx" (20Q57 key: only A is true, so B and "A and B" are wrong). Wrong: "same-state P and D destroys SMJ over a federal counterclaim." Wrong: "unasserted compulsory counterclaim can be brought later if diversity exists."</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1661,27 +1661,27 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Intervention as of right (Rule 24(a)(2))</t>
+          <t>Rule 13: counterclaims</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
+          <t>A counterclaim is a claim against an OPPOSING PARTY (someone already suing you). 13(a) COMPULSORY: arises from the same transaction/occurrence; must be asserted in this suit or it's LOST. 13(b) PERMISSIVE: unrelated; may be asserted but doesn't have to be.</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
+          <t>Who is the target? An opposing party = counterclaim (Rule 13). A non-party who may be liable to YOU for the plaintiff's claim = impleader (Rule 14). Compulsory counterclaims can be forfeited; impleader never is. SMJ: see the Counterclaims and SMJ row.</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
+          <t>Wrong: "counterclaim under Rule 13 against Arman" (not a party; that's impleader, 21Q56). Wrong: "it was them, not us" = counterclaim (it's a DEFENSE, 21Q23). Wrong: "plaintiff is liable on a counterclaim" as a 12(b) ground (21Q15). Wrong: "failing to implead = lost, like a compulsory counterclaim" (21Q22).</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>21Q7, 20Q4</t>
+          <t>21Q56, 21Q22, 21Q23, 21Q15, 20Q16, 20Q57</t>
         </is>
       </c>
     </row>
@@ -1693,27 +1693,27 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Rule 19 (compulsory joinder)</t>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
+          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
+          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
+          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>21Q8, 20Q20</t>
+          <t>21Q7, 20Q4</t>
         </is>
       </c>
     </row>
@@ -1725,27 +1725,27 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Interpleader</t>
+          <t>Rule 19 (compulsory joinder)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
+          <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
+          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Wrong: suing one claimant and impleading the other.</t>
+          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
+          <t>21Q8, 20Q20</t>
         </is>
       </c>
     </row>
@@ -1757,27 +1757,27 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
+          <t>Interpleader</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
+          <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
+          <t>Wrong: suing one claimant and impleading the other.</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
+          <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
         </is>
       </c>
     </row>
@@ -1789,65 +1789,69 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
+          <t>Impleader (Rule 14)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
           <t>Limits on joinder</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F50" s="3" t="inlineStr">
         <is>
           <t>21Q30</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>13. NOT YET COVERED</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Erie (flag: not in Weeks 1-9)</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr"/>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Minimum contacts is a PJ test, not Erie.</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>20Q6, 20Q30</t>
-        </is>
-      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -1857,28 +1861,56 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Forum non conveniens (flag)</t>
+          <t>Erie (flag: not in Weeks 1-9)</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr"/>
       <c r="E52" s="5" t="inlineStr">
         <is>
+          <t>Minimum contacts is a PJ test, not Erie.</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>20Q6, 20Q30</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>13. NOT YET COVERED</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Forum non conveniens (flag)</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
           <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F53" s="5" t="inlineStr">
         <is>
           <t>20Q36</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F52"/>
+  <autoFilter ref="A1:F53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2133,7 +2165,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -2163,7 +2195,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -2283,7 +2315,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2313,7 +2345,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2373,12 +2405,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>43, 45</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>What Rule 12(b) can raise</t>
+          <t>What Rule 12(b) can raise; Rule 13: counterclaims</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2585,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2583,12 +2615,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49, 45</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
+          <t>Impleader (Rule 14); Rule 13: counterclaims</t>
         </is>
       </c>
     </row>
@@ -2613,12 +2645,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49, 45</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
+          <t>Impleader (Rule 14); Rule 13: counterclaims</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2855,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -3153,12 +3185,12 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49, 45</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
+          <t>Impleader (Rule 14); Rule 13: counterclaims</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3215,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -3393,7 +3425,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -3453,7 +3485,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -3573,7 +3605,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -3603,7 +3635,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -3753,12 +3785,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15, 45</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Counterclaims and SMJ</t>
+          <t>Counterclaims and SMJ; Rule 13: counterclaims</t>
         </is>
       </c>
     </row>
@@ -3873,7 +3905,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -3903,7 +3935,7 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -4173,7 +4205,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -4203,7 +4235,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -4353,7 +4385,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>53</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
@@ -4473,7 +4505,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -4983,12 +5015,12 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15, 45</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Counterclaims and SMJ</t>
+          <t>Counterclaims and SMJ; Rule 13: counterclaims</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Civ Pro outline: add Week 8 slide 8 joinder rules summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Index'!$A$1:$F$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1842,44 +1842,44 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Joinder rules at a glance (Week 8 slide 8: Summary of Rules most relevant to Joinder)</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>ADDING A CLAIM, no new party: by plaintiff and generally → Rule 18; by defendant → Rule 13 (counterclaims). ADDING A NEW PARTY and a claim against it (use these INSTEAD of the add-a-claim rules): by plaintiff → Rule 20; by defendant → Rule 14 (impleader). A party MUST be added or plaintiff will lose → Rule 19 (dismissal itself happens under Rule 12, i.e., 12(b)(7)). A party WANTS to join → Rule 24 (intervention). Plaintiff wants the court to resolve ownership of something and bring in at least two other parties → Rule 22 (interpleader). The court consolidates or separates → Rule 42.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Two-step check for ANY joinder: (1) Is it allowed by the joinder rule above? (2) Does it have subject matter jurisdiction? Every addition needs SMJ or it can be dismissed under Rule 12. Original jurisdiction: 28 U.S.C. §1331 (federal question) and §1332 (diversity). Supplemental: 28 U.S.C. §1367.</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: using Rule 18 or 13 when a NEW party is being added (use Rule 20 or 14). Wrong: a standalone "Rule 19 motion" (dismissal is under Rule 12(b)(7)). Wrong: assuming a proper joinder automatically has SMJ.</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>13. NOT YET COVERED</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Erie (flag: not in Weeks 1-9)</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr"/>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Minimum contacts is a PJ test, not Erie.</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>20Q6, 20Q30</t>
-        </is>
-      </c>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -1889,28 +1889,56 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Forum non conveniens (flag)</t>
+          <t>Erie (flag: not in Weeks 1-9)</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr"/>
       <c r="E53" s="5" t="inlineStr">
         <is>
+          <t>Minimum contacts is a PJ test, not Erie.</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>20Q6, 20Q30</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>13. NOT YET COVERED</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Forum non conveniens (flag)</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
           <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>20Q36</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F53"/>
+  <autoFilter ref="A1:F54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3485,7 +3513,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>53</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -4205,7 +4233,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>53</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -4385,7 +4413,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add Week 9 class notes to Civ Pro attack outline
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Index'!$A$1:$F$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1870,75 +1870,363 @@
       <c r="F51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Week 9: the two-step joinder process</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>JOINDER = anything that takes a suit beyond one plaintiff, one defendant, one claim. For EVERY new claim or party, BOTH must be true: (1) the joinder RULE allows the specific thing being attempted (if not, stop there); (2) the court has SUBJECT MATTER JURISDICTION over the new claim.</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>SMJ order: (a) federal question; (b) diversity; (c) supplemental (§1367) only if the new claim is RELATED to the anchor claim. Then make sure no exception applies (§1367(b), §1367(c)). Don't go to supplemental unless you need it. Know which rule goes with which kind of joinder: Rule 18 (P adds claims), Rule 13 (D adds counterclaims), Rule 20 (P adds parties), Rule 14 (D adds parties), Rule 42 (court separates or consolidates).</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: stopping at step 1 ("Rule 18 allows it, so the claim stays"). Some claims can be added procedurally but will be DISMISSED because the court lacks power to hear them. Wrong: running the SMJ analysis when the joinder rule already fails (if Rule 20 doesn't allow it, you're done).</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Rule 18: plaintiff joins claims against one defendant</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Rule 18 is PERMISSIVE and allows EVERYTHING: a plaintiff may join any claims against a defendant, related or unrelated, dependent on each other, or even conflicting. Purpose: efficiency, lumping all claims against one defendant into one suit.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Rule 18 is always a YES; it's never what stops a plaintiff. The limiting factor is SMJ, claim by claim. Class example: federal anchor + state wrongful-discharge claim closely related to it → supplemental jx. Unrelated car-accident claim between same-state parties → no FQ, no diversity, no supplemental (not related to the anchor) → dismissed.</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "Rule 18 bars unrelated claims." Wrong: "joinder of claims is compulsory" (a plaintiff isn't penalized under Rule 18 for leaving a claim out; but statutes of limitations still run, which is one reason to bring everything at once).</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Rule 42: court separates or consolidates</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Rule 42 lets the district judge SEPARATE claims into different trials or CONSOLIDATE cases. The judge keeps power over how complicated a case becomes.</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Exam Q: if the joinder rules are followed AND SMJ is met, can the judge still say no? YES, under Rule 42. A judge is never obligated to let joinder happen.</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "once the rule and SMJ are satisfied, the court must hear the joined claim together."</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Rule 13(a): compulsory counterclaim and forfeiture</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>A pleading MUST state as a counterclaim any claim the pleader has against an opposing party at the time of service if it (A) arises out of the TRANSACTION OR OCCURRENCE that is the subject of the opposing party's claim, and (B) doesn't require adding a party over whom the court can't get jurisdiction.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Same bundle of facts → compulsory. SMJ: a related counterclaim gets SUPPLEMENTAL jx even without FQ or diversity. Forfeiture: if D sits on a compulsory counterclaim and later sues on it in a new federal suit, the original plaintiff argues Rule 13: it was compulsory, so the right to bring it was LOST.</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "D can always bring it later in its own suit." Wrong: confusing this with Rule 18 (plaintiff's claims are never compulsory) or Rule 14 (impleader is never compulsory).</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Rule 13(b): permissive counterclaim and Cordero v. Voltaire</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>PERMISSIVE counterclaim = UNRELATED to the plaintiff's claim. Rule 13 ALLOWS it, but supplemental jx won't work (it needs the same facts), so it must have an INDEPENDENT basis: federal question or diversity.</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Cordero v. Voltaire: no FQ, no diversity, so both counterclaims needed supplemental jx. Counterclaim I arose from the same nucleus of facts as the anchor → compulsory → stays. Counterclaim II came from a different nucleus of facts → permissive → DISMISSED from the federal suit. It isn't necessarily lost: it can be brought in STATE court.</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "permissive counterclaims get supplemental jx." Wrong: "a dismissed permissive counterclaim is forfeited forever."</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>§1367(b) and (c): the exceptions</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>(b): in a case resting only on diversity, no supplemental jx over claims by PLAINTIFFS against persons made parties under Rules 14, 19, 20 or 24 (or claims by would-be Rule 19/24 plaintiffs) when that would be inconsistent with §1332. (c): the court MAY decline supplemental jx, e.g., when the added claims would overwhelm the case.</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>(b) applies only when the PLAINTIFF is adding the party in a diversity-only case. If the DEFENDANT adds a party (Rule 14), (b) doesn't block it. With a federal-question anchor, (b) doesn't apply at all.</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "§1367(b) bars a defendant's impleader of a non-diverse party." Wrong: applying (b) when the anchor is a federal question.</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Rule 20: permissive joinder of parties</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Plaintiffs MAY join (20(a)(1)), and defendants MAY be joined (20(a)(2)), if BOTH: (A) a right to relief jointly, severally or in the alternative arising out of the SAME TRANSACTION, OCCURRENCE, or SERIES of them; AND (B) a QUESTION OF LAW OR FACT COMMON to all.</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Analyze every "arrow" (each P → each D): does Rule 20 allow it, and is there SMJ for it? Class example: P sues D for breach of contract; a friend wants to add an unrelated defamation claim → Rule 20 doesn't allow it (no common facts, no common legal question). Once Rule 20 fails, skip the SMJ analysis.</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>NOTES FIX: the Week 9 notes list the same-transaction + common-question preconditions under Rule 19. Those are Rule 20's elements. Rule 19 is REQUIRED joinder (complete relief / impaired interest / inconsistent obligations), raised by 12(b)(7). Wrong: "Rule 20 joinder is mandatory."</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Mosley v. General Motors (1974)</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Multiple plaintiffs (P1, P2, P3) each suing GM on their OWN federal discrimination claims may join under Rule 20 when their claims arise from the same SERIES of transactions or occurrences and share common questions of law and fact.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>GM's argument: the events were separate, a different nucleus of facts for each plaintiff. The court found common enough questions of fact and law to allow joinder. SMJ: each plaintiff has a federal claim → federal question for every arrow.</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "each plaintiff's injury must come from the exact same event." A series of related transactions can be enough.</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Week 9 in-class hypos: Ann v. Barbara + Charles</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>(1) Ann (IL) sues Barbara (IL) under federal civil-rights law and joins co-worker Charles on a state tort claim (Rule 20 satisfied): YES, supplemental jx. The federal anchor supports §1367(a) jurisdiction over the related state claim, and §1367(b) doesn't apply because the anchor isn't diversity. (2) Ann (IL) sues Barbara (WI) for breach of contract (&gt; $75k, diversity only) and joins Charles (IL) for conspiracy (Rule 20 satisfied): NO. §1367(b) bars a plaintiff's claim against a party joined under Rule 20 when it would destroy complete diversity.</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Same facts, same rule; the anchor decides it. Federal-question anchor → (b) doesn't apply. Diversity-only anchor + plaintiff adds a non-diverse defendant → (b) bars it.</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "supplemental jx works in both because the claims are related." Wrong: "no jx in #1 because Ann and Charles are both from Illinois" (citizenship doesn't matter with a federal anchor).</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>Erie (flag: not in Weeks 1-9)</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr"/>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>Minimum contacts is a PJ test, not Erie.</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t>20Q6, 20Q30</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>Forum non conveniens (flag)</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr"/>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr">
         <is>
           <t>20Q36</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F54"/>
+  <autoFilter ref="A1:F63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3513,7 +3801,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>62</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -4233,7 +4521,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>62</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -4413,7 +4701,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
@@ -5198,7 +5486,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Sources: professor's answer keys/explanations for the 2020 and 2021 finals. Nothing added from outside them.</t>
+          <t>Sources: professor's answer keys/explanations for the 2020 and 2021 finals, the Week 8 joinder slides, and your Week 9 class notes (10/21). Week 9 rows say so in the last column.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Joinder tab to Civ Pro outline (Week 9 class rules only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Attack Outline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Question Index" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Joinder" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Question Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Attack Outline'!$A$1:$F$63</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Question Index'!$A$1:$F$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Question Index'!$A$1:$F$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2237,6 +2238,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What it says</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Example from class</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SMJ check</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>The 2-step process (every joinder)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Joinder = anything that takes a suit beyond 1 plaintiff, 1 defendant, 1 claim. For each new claim or party ask: (1) Does the joinder RULE allow it? If no, stop. (2) Does the court have SMJ? Check federal question → diversity → supplemental (only if related to the anchor claim) → make sure no exception applies.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff adds a claim: Rule 18 says yes (step 1), then check SMJ for that claim (step 2).</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Don't go to supplemental unless you need it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Rule 18: plaintiff adds claims</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A plaintiff may join ANY claims against a defendant: related, unrelated, or even conflicting. Always a yes. Not compulsory.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pam sues her employer under federal law for firing her and adds (a) a state wrongful-discharge claim from the same firing and (b) an unrelated car-accident claim. Rule 18 allows both.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>(a) stays: supplemental (related to the federal anchor). (b) dismissed: no FQ, no diversity, not related.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Rule 13(a): compulsory counterclaim</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Defendant's claim against the plaintiff that arises from the SAME transaction or occurrence. Defendant MUST bring it, or it's lost.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Paula sues Dev over a car collision. Dev doesn't counterclaim for his own injuries. If he sues Paula later, she argues it was compulsory and he forfeited it.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Supplemental (same facts as the anchor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Rule 13(b): permissive counterclaim</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Defendant's claim against the plaintiff that is UNRELATED to the plaintiff's claim. Allowed, not required.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cordero v. Voltaire: Counterclaim I (same facts) = compulsory, stays. Counterclaim II (different facts) = permissive, dismissed. It can still be brought in state court.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Needs its OWN basis: federal question or diversity. No supplemental.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Rule 20: permissive joinder of parties (plaintiff's choice)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>20(a)(1): plaintiffs may join TOGETHER. 20(a)(2): a plaintiff may sue several DEFENDANTS together. BOTH required: (1) same transaction, occurrence, or series; AND (2) a common question of law or fact.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Mosley v. GM: employees at different plants join as plaintiffs over a company-wide policy (allowed). P sues D for breach of contract; a friend wants to add an unrelated defamation claim (NOT allowed; Rule 20 fails, so you never reach SMJ).</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Check SMJ for each "arrow" (each P → each D).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>§1367(b): the diversity exception</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>§1367(c): court may decline</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff piles many state claims onto one small federal claim.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Rule 42: court separates or consolidates</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Even if the joinder rule is met AND there's SMJ, the judge can still separate claims or consolidate cases. The judge is never obligated to let joinder happen.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Six properly joined claims are confusing a jury → judge orders separate trials.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5436,13 +5647,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5472,19 +5683,26 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Question Index: every final question used, with the answer and which outline row(s) it rests on.</t>
+          <t>Joinder: one-page tab with only the joinder rules covered in Week 9 class (10/21), each with a class example.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Orange rows: Erie and forum non conveniens appear on the 2020 final but aren't in your Weeks 1-9 material yet.</t>
+          <t>Question Index: every final question used, with the answer and which outline row(s) it rests on.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Orange rows: Erie and forum non conveniens appear on the 2020 final but aren't in your Weeks 1-9 material yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Sources: professor's answer keys/explanations for the 2020 and 2021 finals, the Week 8 joinder slides, and your Week 9 class notes (10/21). Week 9 rows say so in the last column.</t>
         </is>

</xml_diff>

<commit_message>
Joinder tab: add Rule 22 interpleader and Rule 24 intervention
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -2238,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2382,60 +2382,104 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>§1367(b): the diversity exception</t>
+          <t>Rule 22: interpleader</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+          <t>A party facing DOUBLE OR MULTIPLE LIABILITY to competing claimants can bring them all into one action. (1) By a PLAINTIFF: join the claimants as defendants and require them to interplead. (2) By a DEFENDANT: through a crossclaim or counterclaim. Allowed even if the claims lack a common origin or are adverse and independent, and even if the stakeholder denies owing anyone. Rule 22 supplements Rule 20 and works alongside statutory interpleader (28 U.S.C. §§1335, 1397, 2361).</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+          <t>InsureCo holds a $100,000 life-insurance payout claimed by both the ex-wife and the current wife; it sues both and lets the court decide (plaintiff interpleader). Ana sues BankCo for her late father's account; BankCo brings in a creditor who also claims it (defendant interpleader). An escrow deposit claimed by a buyer and by a contractor under a separate assignment: no common origin, still OK.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+          <t>Still needs SMJ (FQ or diversity) under Rule 22. Statutory interpleader has its own jurisdiction rules (beyond this outline).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>§1367(c): court may decline</t>
+          <t>Rule 24: intervention</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+          <t>A NON-PARTY asks to join. (a) AS OF RIGHT: the court MUST allow a TIMELY motion by anyone with (1) an unconditional statutory right, or (2) an interest in the property or transaction at issue that may be practically impaired, unless existing parties adequately represent it. (b) PERMISSIVE: the court MAY allow a TIMELY motion by anyone with (1) a conditional statutory right, or (2) a claim or defense sharing a common question of law or fact; (b)(2) government officers or agencies may intervene when the case involves a statute or order they administer; (b)(3) the court must consider undue delay or prejudice to the original parties. (c) PROCEDURE: a motion served under Rule 5, with a pleading stating the claim or defense.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Plaintiff piles many state claims onto one small federal claim.</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr"/>
+          <t>An environmental group protecting a wetland at issue: interest + possible impairment + inadequate representation → as of right, but only if timely (waiting 14 months until a week before trial fails). A business with a similar claim against the same defendant → permissive at most; the judge may say no.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Every intervenor's claim still needs SMJ (FQ, diversity, or supplemental, subject to §1367(b) limits).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>§1367(b): the diversity exception</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>§1367(c): court may decline</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff piles many state claims onto one small federal claim.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>Rule 42: court separates or consolidates</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Even if the joinder rule is met AND there's SMJ, the judge can still separate claims or consolidate cases. The judge is never obligated to let joinder happen.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Six properly joined claims are confusing a jury → judge orders separate trials.</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Joinder tab: add casebook interpleader rows (Dunlevy, statutory vs. Rule 22)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -2238,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2397,89 +2397,133 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Still needs SMJ (FQ or diversity) under Rule 22. Statutory interpleader has its own jurisdiction rules (beyond this outline).</t>
+          <t>Still needs SMJ (FQ or diversity) under Rule 22. Statutory interpleader: see the next row.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Rule 24: intervention</t>
+          <t>Interpleader: the stakeholder's dilemma and Dunlevy (casebook p. 825)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>A NON-PARTY asks to join. (a) AS OF RIGHT: the court MUST allow a TIMELY motion by anyone with (1) an unconditional statutory right, or (2) an interest in the property or transaction at issue that may be practically impaired, unless existing parties adequately represent it. (b) PERMISSIVE: the court MAY allow a TIMELY motion by anyone with (1) a conditional statutory right, or (2) a claim or defense sharing a common question of law or fact; (b)(2) government officers or agencies may intervene when the case involves a statute or order they administer; (b)(3) the court must consider undue delay or prejudice to the original parties. (c) PROCEDURE: a motion served under Rule 5, with a pleading stating the claim or defense.</t>
+          <t>The problem: a husband's life insurance policy is payable to "my wife"; the couple divorces, he remarries and dies, and both wives claim the proceeds. If they bring separate suits, both may win. Same situation: two competing claimants each want to withdraw a small business's entire bank account. The stakeholder (insurer or bank) concedes it owes the money but wants a procedure that binds all claimants. Past difficulties: (1) no effective procedural device to join both claimants; (2) possible jurisdictional and venue limitations. INTERPLEADER lets a stakeholder (often a bank or insurer) require the competing claimants to litigate their rights to the fund or property. Rule 22 typifies such a joinder provision, and it allows interpleader even if the stakeholder asserts some claim on the assets itself (e.g., a bank reducing the account balance by an unpaid loan). Typically, the stakeholder invokes interpleader, joining the claimants as parties.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>An environmental group protecting a wetland at issue: interest + possible impairment + inadequate representation → as of right, but only if timely (waiting 14 months until a week before trial fails). A business with a similar claim against the same defendant → permissive at most; the judge may say no.</t>
+          <t>New York Life Insurance Co. v. Dunlevy (1916): Father, in Pennsylvania, bought a policy paying a lump sum after a set number of years. When it came due, Father and Daughter disagreed over who was entitled. Daughter's creditor sued in Pennsylvania; the insurer interpleaded Father, Daughter and Creditor; the Pennsylvania court ruled for Father. Daughter sued the insurer in California. The Supreme Court held the Pennsylvania suit did NOT preclude her claim, because Pennsylvania had not acquired personal jurisdiction over Daughter, who lived in California. The insurer was liable a second time.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Every intervenor's claim still needs SMJ (FQ, diversity, or supplemental, subject to §1367(b) limits).</t>
+          <t>An interpleader proceeding fails to yield a stable resolution if the forum lacks jurisdiction over the claimants (Dunlevy).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>§1367(b): the diversity exception</t>
+          <t>Statutory interpleader (Federal Interpleader Act) vs. Rule 22 (casebook pp. 825-826)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+          <t>Congress responded to Dunlevy-type problems with the Federal Interpleader Act, 28 U.S.C. §§1335, 1397, 2361. The Act: (1) broadens the circumstances in which interpleader is available, eliminating some restrictions older equity doctrines imposed (§1335); (2) removes limitations on federal SMJ (§1335(a)); (3) permits nationwide service of process, interpreted to mean nationwide personal jurisdiction (§2361); (4) expands venue to where any claimant resides (§1397). Rule 22 closely resembles the Act, BUT Rule 22 actions are subject to the NORMAL rules for SMJ (diversity between all plaintiffs and all defendants; amount in controversy), personal jurisdiction (jurisdiction within the state) and venue (residency of all defendants, or where the claim arises).</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+          <t>Dunlevy under the Act: Daughter would be subject to the jurisdiction of the federal courts in Pennsylvania (§2361), which could resolve all the parties' conflicting claims. In practice, Rule 22 is used when the stakeholder is a citizen of one state and all claimants are citizens of a second state: there is no jurisdiction under the Interpleader Act because no two claimants are diverse, but the normal rules for jurisdiction and venue can be satisfied by an action in the state of all claimants.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+          <t>Statutory: SMJ per §1335(a); nationwide PJ (§2361); venue where any claimant resides (§1397). Rule 22: normal SMJ (complete diversity + amount), normal PJ and normal venue.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>§1367(c): court may decline</t>
+          <t>Rule 24: intervention</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+          <t>A NON-PARTY asks to join. (a) AS OF RIGHT: the court MUST allow a TIMELY motion by anyone with (1) an unconditional statutory right, or (2) an interest in the property or transaction at issue that may be practically impaired, unless existing parties adequately represent it. (b) PERMISSIVE: the court MAY allow a TIMELY motion by anyone with (1) a conditional statutory right, or (2) a claim or defense sharing a common question of law or fact; (b)(2) government officers or agencies may intervene when the case involves a statute or order they administer; (b)(3) the court must consider undue delay or prejudice to the original parties. (c) PROCEDURE: a motion served under Rule 5, with a pleading stating the claim or defense.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Plaintiff piles many state claims onto one small federal claim.</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr"/>
+          <t>An environmental group protecting a wetland at issue: interest + possible impairment + inadequate representation → as of right, but only if timely (waiting 14 months until a week before trial fails). A business with a similar claim against the same defendant → permissive at most; the judge may say no.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Every intervenor's claim still needs SMJ (FQ, diversity, or supplemental, subject to §1367(b) limits).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>§1367(b): the diversity exception</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>§1367(c): court may decline</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff piles many state claims onto one small federal claim.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>Rule 42: court separates or consolidates</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Even if the joinder rule is met AND there's SMJ, the judge can still separate claims or consolidate cases. The judge is never obligated to let joinder happen.</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Six properly joined claims are confusing a jury → judge orders separate trials.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Joinder tab: add casebook intervention row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -2238,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2470,60 +2470,78 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>§1367(b): the diversity exception</t>
+          <t>Intervention: purpose, structure and the four Rule 24(a) requirements (casebook intro, through p. 813)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+          <t>PURPOSE: The other joinder devices bring in a party who does NOT want to be there; intervention does the opposite: it lets an unjoined person "elbow her way into a suit where no one wants her." Like compulsory joinder, it flows from the recognition that lawsuits may affect persons not joined. Those effects are not formal preclusion (due process forbids binding one who was not a party), but judgments have broader ripple effects than the decree's formal binding effect. COSTS: existing parties (and perhaps the judge) may be unenthusiastic; intervention complicates and perhaps weakens their strategy (even an intervenor seeking the same outcome has a different perspective and perhaps strategy), may make the suit more expensive and settlement harder, and erodes party autonomy; carried to a logical extreme it turns every lawsuit into a "town meeting." Intervention principles allow some, but not all, who wish to be involved to join. STRUCTURE: (1) INTERVENTION OF RIGHT, Rule 24(a): gives those with STRONG interests the power to insist on joinder; Rule 24(a)(2)'s words echo Rule 19(a)(1)(B) ("an interest relating to . . . the subject of the action . . . so situated that disposing of the action may as a practical matter impair or impede" the would-be intervenor's interests). An applicant who meets Rule 24(a) MUST be allowed to join. (2) PERMISSIVE INTERVENTION, Rule 24(b): the weaker counterpart, for those with weaker bases for insisting on joinder. An applicant who meets only Rule 24(b) MAY be allowed to join; the judge's decision is reviewed only for ABUSE OF DISCRETION. FOUR Rule 24(a) REQUIREMENTS (the focus of most reported cases): (1) TIMELY: the intervenor may not lie in wait until the litigation is on the brink of resolution; (2) an INTEREST in the property or transaction that is the subject of the suit; (3) that interest must be in some strong way AT RISK; (4) even an applicant meeting all of these is denied if those already in the suit ADEQUATELY REPRESENT the interest.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
-        </is>
-      </c>
+          <t>Developer and City Zoning Board litigate whether Developer can build an office building on a plot bordering a residential area. If Developer wins, Homeowner (next to the plot) is affected; if Developer loses, Landowner (owner of another adjacent plot that would be more valuable if commercially developed) is adversely affected. The judgment won't formally bind either, but will affect both, and both might wish to influence the outcome. If entitled to intervene, they would become parties with the right to present evidence and arguments like Developer and the Zoning Board. Next case: NRDC v. U.S. Nuclear Regulatory Commission (10th Cir. 1978): American Mining Congress and Kerr-McGee Nuclear Corp. sought review of the denial of their motions to intervene of right and permissively under Rule 24(a)(2) and (b); the casebook says the case assumes timeliness and analyzes the other three criteria.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>§1367(c): court may decline</t>
+          <t>§1367(b): the diversity exception</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Plaintiff piles many state claims onto one small federal claim.</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr"/>
+          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>§1367(c): court may decline</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff piles many state claims onto one small federal claim.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>Rule 42: court separates or consolidates</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Even if the joinder rule is met AND there's SMJ, the judge can still separate claims or consolidate cases. The judge is never obligated to let joinder happen.</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Six properly joined claims are confusing a jury → judge orders separate trials.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Civ Pro outline: general PJ can exist in many states (with Daimler caution)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1279,44 +1279,44 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>7. GENERAL PJ</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>How many places? (could be all 50 states)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>A corporation can be subject to general jurisdiction anywhere it has continuous and systematic connections, which could theoretically be all fifty states.</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Ask whether its contacts in THIS state are so continuous and systematic that it is essentially at home there. Its state of incorporation and principal place of business always qualify. Caution: the Supreme Court's modern cases (Goodyear 2011; Daimler 2014) say that, outside an "exceptional case," a corporation is at home only in those two places, so "every state where it does a lot of business" rarely works in practice.</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "general jx exists in only one place." Also wrong: treating big sales in a state as automatically enough (Daimler). Contrast diversity citizenship, which is limited to two states at most (row 8).</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>8. SPECIFIC PJ</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>8. SPECIFIC PJ</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Elements</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>(1) Purposeful availment; (2) suit arises out of/relates to the defendant's forum contacts; (3) state interest; (4) reasonableness.</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>All four must be proven when the defendant isn't domiciled in the forum.</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>20Q60, 20Q22</t>
-        </is>
-      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1326,27 +1326,23 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Purposeful availment</t>
+          <t>Elements</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Everything the defendant INTENTIONALLY did in the forum: living there, contracting there, driving its roads, ads aimed at forum residents, banners meant to attract them. A contract clause choosing that state's LAW also counts as evidence (see the Choice-of-LAW clause row).</t>
+          <t>(1) Purposeful availment; (2) suit arises out of/relates to the defendant's forum contacts; (3) state interest; (4) reasonableness.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Purposeful availment doesn't screen related vs. unrelated contacts (that's "arises out of").</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Wrong: "reasonably foreseeable the product would end up there" alone. Minimum contacts is much less than general jx.</t>
-        </is>
-      </c>
+          <t>All four must be proven when the defendant isn't domiciled in the forum.</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>20Q55, 21Q52, 20Q25, 20Q26, 20Q24</t>
+          <t>20Q60, 20Q22</t>
         </is>
       </c>
     </row>
@@ -1358,27 +1354,27 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Arises out of / relates to</t>
+          <t>Purposeful availment</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>The suit springs from or relates to the DEFENDANT'S contacts with the forum.</t>
+          <t>Everything the defendant INTENTIONALLY did in the forum: living there, contracting there, driving its roads, ads aimed at forum residents, banners meant to attract them. A contract clause choosing that state's LAW also counts as evidence (see the Choice-of-LAW clause row).</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Not the plaintiff's contacts.</t>
+          <t>Purposeful availment doesn't screen related vs. unrelated contacts (that's "arises out of").</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "suit sprang from the plaintiff's contacts," "continuous contacts" (general), "a long-arm allows it."</t>
+          <t>Wrong: "reasonably foreseeable the product would end up there" alone. Minimum contacts is much less than general jx.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>21Q36</t>
+          <t>20Q55, 21Q52, 20Q25, 20Q26, 20Q24</t>
         </is>
       </c>
     </row>
@@ -1390,27 +1386,27 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>State interest</t>
+          <t>Arises out of / relates to</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>A state is interested if the plaintiff is from there or the tort occurred there. Being the forum alone isn't enough.</t>
+          <t>The suit springs from or relates to the DEFENDANT'S contacts with the forum.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>The plaintiff's own forum ties can show STATE INTEREST only, never the defendant's contacts. A choice-of-LAW clause can help show state interest (see the Choice-of-LAW clause row).</t>
+          <t>Not the plaintiff's contacts.</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "the forum state is always interested."</t>
+          <t>Wrong: "suit sprang from the plaintiff's contacts," "continuous contacts" (general), "a long-arm allows it."</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>21Q53, 20Q27, 21Q43, 21Q26</t>
+          <t>21Q36</t>
         </is>
       </c>
     </row>
@@ -1422,27 +1418,27 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
+          <t>State interest</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Example: "Any litigation about this contract will be brought in the courts of Illinois." Parties include it to (1) limit exposure to being sued everywhere (e.g., a national company worried about general jx); (2) plan for potential lawsuits by defining where suit can be brought; (3) pick a convenient forum. All are valid reasons.</t>
+          <t>A state is interested if the plaintiff is from there or the tort occurred there. Being the forum alone isn't enough.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>The clause can't override what the forum's long-arm statute requires. Compare the next row: a choice-of-LAW clause says WHICH LAW applies, not where to sue.</t>
+          <t>The plaintiff's own forum ties can show STATE INTEREST only, never the defendant's contacts. A choice-of-LAW clause can help show state interest (see the Choice-of-LAW clause row).</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "these provisions are not enforceable." Choice of FORUM ≠ choice of LAW.</t>
+          <t>Wrong: "the forum state is always interested."</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>21Q25, 20Q32</t>
+          <t>21Q53, 20Q27, 21Q43, 21Q26</t>
         </is>
       </c>
     </row>
@@ -1454,117 +1450,117 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
+          <t>Choice-of-FORUM (forum-selection) clause: WHERE suit is brought</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Example: "Any litigation about this contract will be brought in the courts of Illinois." Parties include it to (1) limit exposure to being sued everywhere (e.g., a national company worried about general jx); (2) plan for potential lawsuits by defining where suit can be brought; (3) pick a convenient forum. All are valid reasons.</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>The clause can't override what the forum's long-arm statute requires. Compare the next row: a choice-of-LAW clause says WHICH LAW applies, not where to sue.</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "these provisions are not enforceable." Choice of FORUM ≠ choice of LAW.</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>21Q25, 20Q32</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>8. SPECIFIC PJ</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
           <t>Choice-of-LAW clause: WHICH STATE'S LAW governs, and what it shows for PJ</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Example: "This contract is to be interpreted under the laws of Wisconsin, regardless of the forum." It picks the governing law, NOT the place of suit. But in a PJ challenge it is evidence for two parts of the constitutional test: (1) the chosen state is INTERESTED in the suit; (2) the party PURPOSEFULLY AVAILED itself of that state.</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Party sued in the chosen-law state and challenging PJ? Use the clause as evidence of STATE INTEREST + PURPOSEFUL AVAILMENT (answer: "A and B"). It's evidence, not consent to jurisdiction there; still run the long-arm and the rest of the test.</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>Wrong: "it establishes TRANSIENT jx" (transient = served while physically present). Wrong: "all of the above" when transient is one of the choices. Wrong: treating it as a choice-of-forum clause.</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>21Q26</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>9. NOTICE / SERVICE</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>9. NOTICE / SERVICE</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Notice standard</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Give as much notice as is reasonable given what you know about each defendant; different defendants may get different notice.</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Known address: serve there. Unknown/pseudonymous: more limited methods.</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Wrong: "publication suffices for both," "no notice to the unknown one," "follow state court rules."</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>21Q16, 20Q1</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>10. VENUE</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>10. VENUE</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>§1391 residence venue</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Venue is proper in any district where any defendant resides IF all defendants reside in the same state.</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Defendants in N.D. Ill. and S.D. Ill.: both districts are proper.</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Where the product was designed or parts made doesn't make venue certain.</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>21Q14, 20Q19</t>
-        </is>
-      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1574,117 +1570,117 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
+          <t>§1391 residence venue</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Venue is proper in any district where any defendant resides IF all defendants reside in the same state.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Defendants in N.D. Ill. and S.D. Ill.: both districts are proper.</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Where the product was designed or parts made doesn't make venue certain.</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>21Q14, 20Q19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>10. VENUE</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
           <t>Dismiss vs. transfer</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Improper venue: dismissal under Rule 12. Even proper venue: transfer to another district (§1404).</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>Venue never sends a case to state court.</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>Wrong: "transfer to state court," "dismiss even though venue is proper."</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>21Q6, 20Q8</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>11. RULE 12 DEFENSES</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>11. RULE 12 DEFENSES</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>What Rule 12(b) can raise</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>No SMJ, no PJ, improper venue, failure to join a Rule 19 party (12(b)(7)).</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>A counterclaim is NOT a Rule 12 defense.</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>Defendant can't argue lack of PJ over the plaintiff.</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>21Q15, 20Q54, 20Q56</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>12. JOINDER</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>12. JOINDER</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Rule 13: counterclaims</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>A counterclaim is a claim against an OPPOSING PARTY (someone already suing you). 13(a) COMPULSORY: arises from the same transaction/occurrence; must be asserted in this suit or it's LOST. 13(b) PERMISSIVE: unrelated; may be asserted but doesn't have to be.</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>Who is the target? An opposing party = counterclaim (Rule 13). A non-party who may be liable to YOU for the plaintiff's claim = impleader (Rule 14). Compulsory counterclaims can be forfeited; impleader never is. SMJ: see the Counterclaims and SMJ row.</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Wrong: "counterclaim under Rule 13 against Arman" (not a party; that's impleader, 21Q56). Wrong: "it was them, not us" = counterclaim (it's a DEFENSE, 21Q23). Wrong: "plaintiff is liable on a counterclaim" as a 12(b) ground (21Q15). Wrong: "failing to implead = lost, like a compulsory counterclaim" (21Q22).</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>21Q56, 21Q22, 21Q23, 21Q15, 20Q16, 20Q57</t>
-        </is>
-      </c>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -1694,27 +1690,27 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Intervention as of right (Rule 24(a)(2))</t>
+          <t>Rule 13: counterclaims</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
+          <t>A counterclaim is a claim against an OPPOSING PARTY (someone already suing you). 13(a) COMPULSORY: arises from the same transaction/occurrence; must be asserted in this suit or it's LOST. 13(b) PERMISSIVE: unrelated; may be asserted but doesn't have to be.</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
+          <t>Who is the target? An opposing party = counterclaim (Rule 13). A non-party who may be liable to YOU for the plaintiff's claim = impleader (Rule 14). Compulsory counterclaims can be forfeited; impleader never is. SMJ: see the Counterclaims and SMJ row.</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
+          <t>Wrong: "counterclaim under Rule 13 against Arman" (not a party; that's impleader, 21Q56). Wrong: "it was them, not us" = counterclaim (it's a DEFENSE, 21Q23). Wrong: "plaintiff is liable on a counterclaim" as a 12(b) ground (21Q15). Wrong: "failing to implead = lost, like a compulsory counterclaim" (21Q22).</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>21Q7, 20Q4</t>
+          <t>21Q56, 21Q22, 21Q23, 21Q15, 20Q16, 20Q57</t>
         </is>
       </c>
     </row>
@@ -1726,27 +1722,27 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Rule 19 (compulsory joinder)</t>
+          <t>Intervention as of right (Rule 24(a)(2))</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
+          <t>ALL FOUR required: (1) TIMELY motion; (2) interest relating to the subject of the suit; (3) disposition may IMPAIR or impede that interest; (4) existing parties don't ADEQUATELY REPRESENT it.</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
+          <t>Check timeliness FIRST: how long since the would-be intervenor knew of the suit, and how close to trial? Failing ANY one element (e.g., waiting 14 months until a week before trial) = DENIED, even if interest + inadequate representation are clear.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
+          <t>Wrong: "granted: interest + inadequate representation is enough" (ignores timeliness). Wrong: "can intervene because of diversity." Wrong: "only plaintiffs can intervene."</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>21Q8, 20Q20</t>
+          <t>21Q7, 20Q4</t>
         </is>
       </c>
     </row>
@@ -1758,27 +1754,27 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Interpleader</t>
+          <t>Rule 19 (compulsory joinder)</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
+          <t>A missing required party is raised by a Rule 12(b)(7) motion to dismiss for failure to join under Rule 19.</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
+          <t>Example: Lathrop's exclusive-supplier conflict between Corynna and Hallwein.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Wrong: suing one claimant and impleading the other.</t>
+          <t>Wrong: a standalone "Rule 19 motion," impleader (Rule 14), or a 12(b)(1) SMJ motion.</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
+          <t>21Q8, 20Q20</t>
         </is>
       </c>
     </row>
@@ -1790,27 +1786,27 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Impleader (Rule 14)</t>
+          <t>Interpleader</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
+          <t>A stakeholder facing competing claims (return it to A, B sues; return to B, A sues; keep it, both sue) brings interpleader against all claimants.</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+          <t>Connection to Rule 19: interpleader brings all the would-be compulsory parties in at once.</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
+          <t>Wrong: suing one claimant and impleading the other.</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
+          <t>21Q12, 21Q13, 20Q10, 20Q11, 20Q21</t>
         </is>
       </c>
     </row>
@@ -1822,23 +1818,27 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Limits on joinder</t>
+          <t>Impleader (Rule 14)</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr"/>
+          <t>Defendant brings in a third party who may be liable TO THE DEFENDANT for the plaintiff's claim. The legal connection must already exist (contract/indemnity, insurance, implied warranty, contribution); impleader doesn't create it.</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+        </is>
+      </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
+          <t>Wrong: "implead both suppliers since one must be at fault." Wrong: "insurer is a Rule 19 necessary party."</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>21Q30</t>
+          <t>21Q21, 21Q22, 21Q23, 21Q56, 21Q57, 20Q31, 20Q40</t>
         </is>
       </c>
     </row>
@@ -1850,25 +1850,25 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Joinder rules at a glance (Week 8 slide 8: Summary of Rules most relevant to Joinder)</t>
+          <t>Limits on joinder</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>ADDING A CLAIM, no new party: by plaintiff and generally → Rule 18; by defendant → Rule 13 (counterclaims). ADDING A NEW PARTY and a claim against it (use these INSTEAD of the add-a-claim rules): by plaintiff → Rule 20; by defendant → Rule 14 (impleader). A party MUST be added or plaintiff will lose → Rule 19 (dismissal itself happens under Rule 12, i.e., 12(b)(7)). A party WANTS to join → Rule 24 (intervention). Plaintiff wants the court to resolve ownership of something and bring in at least two other parties → Rule 22 (interpleader). The court consolidates or separates → Rule 42.</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>Two-step check for ANY joinder: (1) Is it allowed by the joinder rule above? (2) Does it have subject matter jurisdiction? Every addition needs SMJ or it can be dismissed under Rule 12. Original jurisdiction: 28 U.S.C. §1331 (federal question) and §1332 (diversity). Supplemental: 28 U.S.C. §1367.</t>
-        </is>
-      </c>
+          <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Wrong: using Rule 18 or 13 when a NEW party is being added (use Rule 20 or 14). Wrong: a standalone "Rule 19 motion" (dismissal is under Rule 12(b)(7)). Wrong: assuming a proper joinder automatically has SMJ.</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr"/>
+          <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>21Q30</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -1878,29 +1878,25 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Week 9: the two-step joinder process</t>
+          <t>Joinder rules at a glance (Week 8 slide 8: Summary of Rules most relevant to Joinder)</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>JOINDER = anything that takes a suit beyond one plaintiff, one defendant, one claim. For EVERY new claim or party, BOTH must be true: (1) the joinder RULE allows the specific thing being attempted (if not, stop there); (2) the court has SUBJECT MATTER JURISDICTION over the new claim.</t>
+          <t>ADDING A CLAIM, no new party: by plaintiff and generally → Rule 18; by defendant → Rule 13 (counterclaims). ADDING A NEW PARTY and a claim against it (use these INSTEAD of the add-a-claim rules): by plaintiff → Rule 20; by defendant → Rule 14 (impleader). A party MUST be added or plaintiff will lose → Rule 19 (dismissal itself happens under Rule 12, i.e., 12(b)(7)). A party WANTS to join → Rule 24 (intervention). Plaintiff wants the court to resolve ownership of something and bring in at least two other parties → Rule 22 (interpleader). The court consolidates or separates → Rule 42.</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>SMJ order: (a) federal question; (b) diversity; (c) supplemental (§1367) only if the new claim is RELATED to the anchor claim. Then make sure no exception applies (§1367(b), §1367(c)). Don't go to supplemental unless you need it. Know which rule goes with which kind of joinder: Rule 18 (P adds claims), Rule 13 (D adds counterclaims), Rule 20 (P adds parties), Rule 14 (D adds parties), Rule 42 (court separates or consolidates).</t>
+          <t>Two-step check for ANY joinder: (1) Is it allowed by the joinder rule above? (2) Does it have subject matter jurisdiction? Every addition needs SMJ or it can be dismissed under Rule 12. Original jurisdiction: 28 U.S.C. §1331 (federal question) and §1332 (diversity). Supplemental: 28 U.S.C. §1367.</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Wrong: stopping at step 1 ("Rule 18 allows it, so the claim stays"). Some claims can be added procedurally but will be DISMISSED because the court lacks power to hear them. Wrong: running the SMJ analysis when the joinder rule already fails (if Rule 20 doesn't allow it, you're done).</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>Week 9 class notes (10/21)</t>
-        </is>
-      </c>
+          <t>Wrong: using Rule 18 or 13 when a NEW party is being added (use Rule 20 or 14). Wrong: a standalone "Rule 19 motion" (dismissal is under Rule 12(b)(7)). Wrong: assuming a proper joinder automatically has SMJ.</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -1910,22 +1906,22 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Rule 18: plaintiff joins claims against one defendant</t>
+          <t>Week 9: the two-step joinder process</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Rule 18 is PERMISSIVE and allows EVERYTHING: a plaintiff may join any claims against a defendant, related or unrelated, dependent on each other, or even conflicting. Purpose: efficiency, lumping all claims against one defendant into one suit.</t>
+          <t>JOINDER = anything that takes a suit beyond one plaintiff, one defendant, one claim. For EVERY new claim or party, BOTH must be true: (1) the joinder RULE allows the specific thing being attempted (if not, stop there); (2) the court has SUBJECT MATTER JURISDICTION over the new claim.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Rule 18 is always a YES; it's never what stops a plaintiff. The limiting factor is SMJ, claim by claim. Class example: federal anchor + state wrongful-discharge claim closely related to it → supplemental jx. Unrelated car-accident claim between same-state parties → no FQ, no diversity, no supplemental (not related to the anchor) → dismissed.</t>
+          <t>SMJ order: (a) federal question; (b) diversity; (c) supplemental (§1367) only if the new claim is RELATED to the anchor claim. Then make sure no exception applies (§1367(b), §1367(c)). Don't go to supplemental unless you need it. Know which rule goes with which kind of joinder: Rule 18 (P adds claims), Rule 13 (D adds counterclaims), Rule 20 (P adds parties), Rule 14 (D adds parties), Rule 42 (court separates or consolidates).</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "Rule 18 bars unrelated claims." Wrong: "joinder of claims is compulsory" (a plaintiff isn't penalized under Rule 18 for leaving a claim out; but statutes of limitations still run, which is one reason to bring everything at once).</t>
+          <t>Wrong: stopping at step 1 ("Rule 18 allows it, so the claim stays"). Some claims can be added procedurally but will be DISMISSED because the court lacks power to hear them. Wrong: running the SMJ analysis when the joinder rule already fails (if Rule 20 doesn't allow it, you're done).</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -1942,22 +1938,22 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Rule 42: court separates or consolidates</t>
+          <t>Rule 18: plaintiff joins claims against one defendant</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Rule 42 lets the district judge SEPARATE claims into different trials or CONSOLIDATE cases. The judge keeps power over how complicated a case becomes.</t>
+          <t>Rule 18 is PERMISSIVE and allows EVERYTHING: a plaintiff may join any claims against a defendant, related or unrelated, dependent on each other, or even conflicting. Purpose: efficiency, lumping all claims against one defendant into one suit.</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Exam Q: if the joinder rules are followed AND SMJ is met, can the judge still say no? YES, under Rule 42. A judge is never obligated to let joinder happen.</t>
+          <t>Rule 18 is always a YES; it's never what stops a plaintiff. The limiting factor is SMJ, claim by claim. Class example: federal anchor + state wrongful-discharge claim closely related to it → supplemental jx. Unrelated car-accident claim between same-state parties → no FQ, no diversity, no supplemental (not related to the anchor) → dismissed.</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "once the rule and SMJ are satisfied, the court must hear the joined claim together."</t>
+          <t>Wrong: "Rule 18 bars unrelated claims." Wrong: "joinder of claims is compulsory" (a plaintiff isn't penalized under Rule 18 for leaving a claim out; but statutes of limitations still run, which is one reason to bring everything at once).</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -1974,22 +1970,22 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Rule 13(a): compulsory counterclaim and forfeiture</t>
+          <t>Rule 42: court separates or consolidates</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>A pleading MUST state as a counterclaim any claim the pleader has against an opposing party at the time of service if it (A) arises out of the TRANSACTION OR OCCURRENCE that is the subject of the opposing party's claim, and (B) doesn't require adding a party over whom the court can't get jurisdiction.</t>
+          <t>Rule 42 lets the district judge SEPARATE claims into different trials or CONSOLIDATE cases. The judge keeps power over how complicated a case becomes.</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Same bundle of facts → compulsory. SMJ: a related counterclaim gets SUPPLEMENTAL jx even without FQ or diversity. Forfeiture: if D sits on a compulsory counterclaim and later sues on it in a new federal suit, the original plaintiff argues Rule 13: it was compulsory, so the right to bring it was LOST.</t>
+          <t>Exam Q: if the joinder rules are followed AND SMJ is met, can the judge still say no? YES, under Rule 42. A judge is never obligated to let joinder happen.</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "D can always bring it later in its own suit." Wrong: confusing this with Rule 18 (plaintiff's claims are never compulsory) or Rule 14 (impleader is never compulsory).</t>
+          <t>Wrong: "once the rule and SMJ are satisfied, the court must hear the joined claim together."</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -2006,22 +2002,22 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Rule 13(b): permissive counterclaim and Cordero v. Voltaire</t>
+          <t>Rule 13(a): compulsory counterclaim and forfeiture</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>PERMISSIVE counterclaim = UNRELATED to the plaintiff's claim. Rule 13 ALLOWS it, but supplemental jx won't work (it needs the same facts), so it must have an INDEPENDENT basis: federal question or diversity.</t>
+          <t>A pleading MUST state as a counterclaim any claim the pleader has against an opposing party at the time of service if it (A) arises out of the TRANSACTION OR OCCURRENCE that is the subject of the opposing party's claim, and (B) doesn't require adding a party over whom the court can't get jurisdiction.</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Cordero v. Voltaire: no FQ, no diversity, so both counterclaims needed supplemental jx. Counterclaim I arose from the same nucleus of facts as the anchor → compulsory → stays. Counterclaim II came from a different nucleus of facts → permissive → DISMISSED from the federal suit. It isn't necessarily lost: it can be brought in STATE court.</t>
+          <t>Same bundle of facts → compulsory. SMJ: a related counterclaim gets SUPPLEMENTAL jx even without FQ or diversity. Forfeiture: if D sits on a compulsory counterclaim and later sues on it in a new federal suit, the original plaintiff argues Rule 13: it was compulsory, so the right to bring it was LOST.</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "permissive counterclaims get supplemental jx." Wrong: "a dismissed permissive counterclaim is forfeited forever."</t>
+          <t>Wrong: "D can always bring it later in its own suit." Wrong: confusing this with Rule 18 (plaintiff's claims are never compulsory) or Rule 14 (impleader is never compulsory).</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2038,22 +2034,22 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>§1367(b) and (c): the exceptions</t>
+          <t>Rule 13(b): permissive counterclaim and Cordero v. Voltaire</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>(b): in a case resting only on diversity, no supplemental jx over claims by PLAINTIFFS against persons made parties under Rules 14, 19, 20 or 24 (or claims by would-be Rule 19/24 plaintiffs) when that would be inconsistent with §1332. (c): the court MAY decline supplemental jx, e.g., when the added claims would overwhelm the case.</t>
+          <t>PERMISSIVE counterclaim = UNRELATED to the plaintiff's claim. Rule 13 ALLOWS it, but supplemental jx won't work (it needs the same facts), so it must have an INDEPENDENT basis: federal question or diversity.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>(b) applies only when the PLAINTIFF is adding the party in a diversity-only case. If the DEFENDANT adds a party (Rule 14), (b) doesn't block it. With a federal-question anchor, (b) doesn't apply at all.</t>
+          <t>Cordero v. Voltaire: no FQ, no diversity, so both counterclaims needed supplemental jx. Counterclaim I arose from the same nucleus of facts as the anchor → compulsory → stays. Counterclaim II came from a different nucleus of facts → permissive → DISMISSED from the federal suit. It isn't necessarily lost: it can be brought in STATE court.</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "§1367(b) bars a defendant's impleader of a non-diverse party." Wrong: applying (b) when the anchor is a federal question.</t>
+          <t>Wrong: "permissive counterclaims get supplemental jx." Wrong: "a dismissed permissive counterclaim is forfeited forever."</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -2070,22 +2066,22 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Rule 20: permissive joinder of parties</t>
+          <t>§1367(b) and (c): the exceptions</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Plaintiffs MAY join (20(a)(1)), and defendants MAY be joined (20(a)(2)), if BOTH: (A) a right to relief jointly, severally or in the alternative arising out of the SAME TRANSACTION, OCCURRENCE, or SERIES of them; AND (B) a QUESTION OF LAW OR FACT COMMON to all.</t>
+          <t>(b): in a case resting only on diversity, no supplemental jx over claims by PLAINTIFFS against persons made parties under Rules 14, 19, 20 or 24 (or claims by would-be Rule 19/24 plaintiffs) when that would be inconsistent with §1332. (c): the court MAY decline supplemental jx, e.g., when the added claims would overwhelm the case.</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Analyze every "arrow" (each P → each D): does Rule 20 allow it, and is there SMJ for it? Class example: P sues D for breach of contract; a friend wants to add an unrelated defamation claim → Rule 20 doesn't allow it (no common facts, no common legal question). Once Rule 20 fails, skip the SMJ analysis.</t>
+          <t>(b) applies only when the PLAINTIFF is adding the party in a diversity-only case. If the DEFENDANT adds a party (Rule 14), (b) doesn't block it. With a federal-question anchor, (b) doesn't apply at all.</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>NOTES FIX: the Week 9 notes list the same-transaction + common-question preconditions under Rule 19. Those are Rule 20's elements. Rule 19 is REQUIRED joinder (complete relief / impaired interest / inconsistent obligations), raised by 12(b)(7). Wrong: "Rule 20 joinder is mandatory."</t>
+          <t>Wrong: "§1367(b) bars a defendant's impleader of a non-diverse party." Wrong: applying (b) when the anchor is a federal question.</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -2102,22 +2098,22 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Mosley v. General Motors (1974)</t>
+          <t>Rule 20: permissive joinder of parties</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Multiple plaintiffs (P1, P2, P3) each suing GM on their OWN federal discrimination claims may join under Rule 20 when their claims arise from the same SERIES of transactions or occurrences and share common questions of law and fact.</t>
+          <t>Plaintiffs MAY join (20(a)(1)), and defendants MAY be joined (20(a)(2)), if BOTH: (A) a right to relief jointly, severally or in the alternative arising out of the SAME TRANSACTION, OCCURRENCE, or SERIES of them; AND (B) a QUESTION OF LAW OR FACT COMMON to all.</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>GM's argument: the events were separate, a different nucleus of facts for each plaintiff. The court found common enough questions of fact and law to allow joinder. SMJ: each plaintiff has a federal claim → federal question for every arrow.</t>
+          <t>Analyze every "arrow" (each P → each D): does Rule 20 allow it, and is there SMJ for it? Class example: P sues D for breach of contract; a friend wants to add an unrelated defamation claim → Rule 20 doesn't allow it (no common facts, no common legal question). Once Rule 20 fails, skip the SMJ analysis.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "each plaintiff's injury must come from the exact same event." A series of related transactions can be enough.</t>
+          <t>NOTES FIX: the Week 9 notes list the same-transaction + common-question preconditions under Rule 19. Those are Rule 20's elements. Rule 19 is REQUIRED joinder (complete relief / impaired interest / inconsistent obligations), raised by 12(b)(7). Wrong: "Rule 20 joinder is mandatory."</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -2134,69 +2130,73 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
+          <t>Mosley v. General Motors (1974)</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Multiple plaintiffs (P1, P2, P3) each suing GM on their OWN federal discrimination claims may join under Rule 20 when their claims arise from the same SERIES of transactions or occurrences and share common questions of law and fact.</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>GM's argument: the events were separate, a different nucleus of facts for each plaintiff. The court found common enough questions of fact and law to allow joinder. SMJ: each plaintiff has a federal claim → federal question for every arrow.</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "each plaintiff's injury must come from the exact same event." A series of related transactions can be enough.</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
           <t>Week 9 in-class hypos: Ann v. Barbara + Charles</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>(1) Ann (IL) sues Barbara (IL) under federal civil-rights law and joins co-worker Charles on a state tort claim (Rule 20 satisfied): YES, supplemental jx. The federal anchor supports §1367(a) jurisdiction over the related state claim, and §1367(b) doesn't apply because the anchor isn't diversity. (2) Ann (IL) sues Barbara (WI) for breach of contract (&gt; $75k, diversity only) and joins Charles (IL) for conspiracy (Rule 20 satisfied): NO. §1367(b) bars a plaintiff's claim against a party joined under Rule 20 when it would destroy complete diversity.</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>Same facts, same rule; the anchor decides it. Federal-question anchor → (b) doesn't apply. Diversity-only anchor + plaintiff adds a non-diverse defendant → (b) bars it.</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>Wrong: "supplemental jx works in both because the claims are related." Wrong: "no jx in #1 because Ann and Charles are both from Illinois" (citizenship doesn't matter with a federal anchor).</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>Week 9 class notes (10/21)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>13. NOT YET COVERED</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>Erie (flag: not in Weeks 1-9)</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="inlineStr">
-        <is>
-          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr"/>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>Minimum contacts is a PJ test, not Erie.</t>
-        </is>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>20Q6, 20Q30</t>
-        </is>
-      </c>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -2206,21 +2206,49 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Forum non conveniens (flag)</t>
+          <t>Erie (flag: not in Weeks 1-9)</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr"/>
       <c r="E63" s="5" t="inlineStr">
         <is>
+          <t>Minimum contacts is a PJ test, not Erie.</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>20Q6, 20Q30</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>13. NOT YET COVERED</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Forum non conveniens (flag)</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr"/>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
           <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t>20Q36</t>
         </is>

</xml_diff>

<commit_message>
Civ Pro outline: add Week 10 (10/28) joinder notes
Adds a Rule 14 impleader row and a third-party-defendant counterclaim
row to the Joinder tab, expands the §1367(c) row (novel state-law
issue, Rule 42 alternative, how a party resists joinder), adds a
Week 10 row to the Attack Outline, and corrects the Question Index
row references.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Civ_Pro_Attack_Outline.xlsx
+++ b/Civ_Pro_Attack_Outline.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Impleader is NEVER compulsory. "It was him, not me" is a DEFENSE, not impleader.</t>
+          <t>Impleader is NEVER compulsory: the defendant can sue the third party later in a separate suit. "It was him, not me" is a DEFENSE, not impleader.</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -1850,23 +1850,27 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Limits on joinder</t>
+          <t>Week 10: third-party defendant's counterclaims; resisting joinder</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr"/>
+          <t>A third-party defendant may counterclaim against the defendant who impleaded it (Rule 13); related or unrelated, the rule allows it. A party resisting joinder argues no SMJ, or asks the court to decline supplemental jx under §1367(c) (novel state-law issue; added claims would overwhelm the case).</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Run both steps for the counterclaim: rule (always yes) → SMJ (FQ, diversity, or supplemental if related). §1367(c) comes up only if the claim rests on supplemental jx.</t>
+        </is>
+      </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
+          <t>Wrong: 'a third-party defendant can't counterclaim.' Wrong: 'an unrelated counterclaim gets supplemental jx.' Wrong: invoking §1367(c) against a claim that has its own diversity or FQ basis.</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>21Q30</t>
+          <t>Week 10 class notes (10/28)</t>
         </is>
       </c>
     </row>
@@ -1878,25 +1882,25 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Joinder rules at a glance (Week 8 slide 8: Summary of Rules most relevant to Joinder)</t>
+          <t>Limits on joinder</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>ADDING A CLAIM, no new party: by plaintiff and generally → Rule 18; by defendant → Rule 13 (counterclaims). ADDING A NEW PARTY and a claim against it (use these INSTEAD of the add-a-claim rules): by plaintiff → Rule 20; by defendant → Rule 14 (impleader). A party MUST be added or plaintiff will lose → Rule 19 (dismissal itself happens under Rule 12, i.e., 12(b)(7)). A party WANTS to join → Rule 24 (intervention). Plaintiff wants the court to resolve ownership of something and bring in at least two other parties → Rule 22 (interpleader). The court consolidates or separates → Rule 42.</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Two-step check for ANY joinder: (1) Is it allowed by the joinder rule above? (2) Does it have subject matter jurisdiction? Every addition needs SMJ or it can be dismissed under Rule 12. Original jurisdiction: 28 U.S.C. §1331 (federal question) and §1332 (diversity). Supplemental: 28 U.S.C. §1367.</t>
-        </is>
-      </c>
+          <t>No set limit on the number of claims or parties; the judge can sever or separate if it gets too complex.</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr"/>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Wrong: using Rule 18 or 13 when a NEW party is being added (use Rule 20 or 14). Wrong: a standalone "Rule 19 motion" (dismissal is under Rule 12(b)(7)). Wrong: assuming a proper joinder automatically has SMJ.</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr"/>
+          <t>Wrong: "maximum of 2 joinders," "one joinder per litigant."</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>21Q30</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -1906,29 +1910,25 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Week 9: the two-step joinder process</t>
+          <t>Joinder rules at a glance (Week 8 slide 8: Summary of Rules most relevant to Joinder)</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>JOINDER = anything that takes a suit beyond one plaintiff, one defendant, one claim. For EVERY new claim or party, BOTH must be true: (1) the joinder RULE allows the specific thing being attempted (if not, stop there); (2) the court has SUBJECT MATTER JURISDICTION over the new claim.</t>
+          <t>ADDING A CLAIM, no new party: by plaintiff and generally → Rule 18; by defendant → Rule 13 (counterclaims). ADDING A NEW PARTY and a claim against it (use these INSTEAD of the add-a-claim rules): by plaintiff → Rule 20; by defendant → Rule 14 (impleader). A party MUST be added or plaintiff will lose → Rule 19 (dismissal itself happens under Rule 12, i.e., 12(b)(7)). A party WANTS to join → Rule 24 (intervention). Plaintiff wants the court to resolve ownership of something and bring in at least two other parties → Rule 22 (interpleader). The court consolidates or separates → Rule 42.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>SMJ order: (a) federal question; (b) diversity; (c) supplemental (§1367) only if the new claim is RELATED to the anchor claim. Then make sure no exception applies (§1367(b), §1367(c)). Don't go to supplemental unless you need it. Know which rule goes with which kind of joinder: Rule 18 (P adds claims), Rule 13 (D adds counterclaims), Rule 20 (P adds parties), Rule 14 (D adds parties), Rule 42 (court separates or consolidates).</t>
+          <t>Two-step check for ANY joinder: (1) Is it allowed by the joinder rule above? (2) Does it have subject matter jurisdiction? Every addition needs SMJ or it can be dismissed under Rule 12. Original jurisdiction: 28 U.S.C. §1331 (federal question) and §1332 (diversity). Supplemental: 28 U.S.C. §1367.</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Wrong: stopping at step 1 ("Rule 18 allows it, so the claim stays"). Some claims can be added procedurally but will be DISMISSED because the court lacks power to hear them. Wrong: running the SMJ analysis when the joinder rule already fails (if Rule 20 doesn't allow it, you're done).</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>Week 9 class notes (10/21)</t>
-        </is>
-      </c>
+          <t>Wrong: using Rule 18 or 13 when a NEW party is being added (use Rule 20 or 14). Wrong: a standalone "Rule 19 motion" (dismissal is under Rule 12(b)(7)). Wrong: assuming a proper joinder automatically has SMJ.</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Rule 18: plaintiff joins claims against one defendant</t>
+          <t>Week 9: the two-step joinder process</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Rule 18 is PERMISSIVE and allows EVERYTHING: a plaintiff may join any claims against a defendant, related or unrelated, dependent on each other, or even conflicting. Purpose: efficiency, lumping all claims against one defendant into one suit.</t>
+          <t>JOINDER = anything that takes a suit beyond one plaintiff, one defendant, one claim. For EVERY new claim or party, BOTH must be true: (1) the joinder RULE allows the specific thing being attempted (if not, stop there); (2) the court has SUBJECT MATTER JURISDICTION over the new claim.</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Rule 18 is always a YES; it's never what stops a plaintiff. The limiting factor is SMJ, claim by claim. Class example: federal anchor + state wrongful-discharge claim closely related to it → supplemental jx. Unrelated car-accident claim between same-state parties → no FQ, no diversity, no supplemental (not related to the anchor) → dismissed.</t>
+          <t>SMJ order: (a) federal question; (b) diversity; (c) supplemental (§1367) only if the new claim is RELATED to the anchor claim. Then make sure no exception applies (§1367(b), §1367(c)). Don't go to supplemental unless you need it. Know which rule goes with which kind of joinder: Rule 18 (P adds claims), Rule 13 (D adds counterclaims), Rule 20 (P adds parties), Rule 14 (D adds parties), Rule 42 (court separates or consolidates).</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "Rule 18 bars unrelated claims." Wrong: "joinder of claims is compulsory" (a plaintiff isn't penalized under Rule 18 for leaving a claim out; but statutes of limitations still run, which is one reason to bring everything at once).</t>
+          <t>Wrong: stopping at step 1 ("Rule 18 allows it, so the claim stays"). Some claims can be added procedurally but will be DISMISSED because the court lacks power to hear them. Wrong: running the SMJ analysis when the joinder rule already fails (if Rule 20 doesn't allow it, you're done).</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -1970,22 +1970,22 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Rule 42: court separates or consolidates</t>
+          <t>Rule 18: plaintiff joins claims against one defendant</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Rule 42 lets the district judge SEPARATE claims into different trials or CONSOLIDATE cases. The judge keeps power over how complicated a case becomes.</t>
+          <t>Rule 18 is PERMISSIVE and allows EVERYTHING: a plaintiff may join any claims against a defendant, related or unrelated, dependent on each other, or even conflicting. Purpose: efficiency, lumping all claims against one defendant into one suit.</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Exam Q: if the joinder rules are followed AND SMJ is met, can the judge still say no? YES, under Rule 42. A judge is never obligated to let joinder happen.</t>
+          <t>Rule 18 is always a YES; it's never what stops a plaintiff. The limiting factor is SMJ, claim by claim. Class example: federal anchor + state wrongful-discharge claim closely related to it → supplemental jx. Unrelated car-accident claim between same-state parties → no FQ, no diversity, no supplemental (not related to the anchor) → dismissed.</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "once the rule and SMJ are satisfied, the court must hear the joined claim together."</t>
+          <t>Wrong: "Rule 18 bars unrelated claims." Wrong: "joinder of claims is compulsory" (a plaintiff isn't penalized under Rule 18 for leaving a claim out; but statutes of limitations still run, which is one reason to bring everything at once).</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -2002,22 +2002,22 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Rule 13(a): compulsory counterclaim and forfeiture</t>
+          <t>Rule 42: court separates or consolidates</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>A pleading MUST state as a counterclaim any claim the pleader has against an opposing party at the time of service if it (A) arises out of the TRANSACTION OR OCCURRENCE that is the subject of the opposing party's claim, and (B) doesn't require adding a party over whom the court can't get jurisdiction.</t>
+          <t>Rule 42 lets the district judge SEPARATE claims into different trials or CONSOLIDATE cases. The judge keeps power over how complicated a case becomes.</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Same bundle of facts → compulsory. SMJ: a related counterclaim gets SUPPLEMENTAL jx even without FQ or diversity. Forfeiture: if D sits on a compulsory counterclaim and later sues on it in a new federal suit, the original plaintiff argues Rule 13: it was compulsory, so the right to bring it was LOST.</t>
+          <t>Exam Q: if the joinder rules are followed AND SMJ is met, can the judge still say no? YES, under Rule 42. A judge is never obligated to let joinder happen.</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "D can always bring it later in its own suit." Wrong: confusing this with Rule 18 (plaintiff's claims are never compulsory) or Rule 14 (impleader is never compulsory).</t>
+          <t>Wrong: "once the rule and SMJ are satisfied, the court must hear the joined claim together."</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2034,22 +2034,22 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Rule 13(b): permissive counterclaim and Cordero v. Voltaire</t>
+          <t>Rule 13(a): compulsory counterclaim and forfeiture</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>PERMISSIVE counterclaim = UNRELATED to the plaintiff's claim. Rule 13 ALLOWS it, but supplemental jx won't work (it needs the same facts), so it must have an INDEPENDENT basis: federal question or diversity.</t>
+          <t>A pleading MUST state as a counterclaim any claim the pleader has against an opposing party at the time of service if it (A) arises out of the TRANSACTION OR OCCURRENCE that is the subject of the opposing party's claim, and (B) doesn't require adding a party over whom the court can't get jurisdiction.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Cordero v. Voltaire: no FQ, no diversity, so both counterclaims needed supplemental jx. Counterclaim I arose from the same nucleus of facts as the anchor → compulsory → stays. Counterclaim II came from a different nucleus of facts → permissive → DISMISSED from the federal suit. It isn't necessarily lost: it can be brought in STATE court.</t>
+          <t>Same bundle of facts → compulsory. SMJ: a related counterclaim gets SUPPLEMENTAL jx even without FQ or diversity. Forfeiture: if D sits on a compulsory counterclaim and later sues on it in a new federal suit, the original plaintiff argues Rule 13: it was compulsory, so the right to bring it was LOST.</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "permissive counterclaims get supplemental jx." Wrong: "a dismissed permissive counterclaim is forfeited forever."</t>
+          <t>Wrong: "D can always bring it later in its own suit." Wrong: confusing this with Rule 18 (plaintiff's claims are never compulsory) or Rule 14 (impleader is never compulsory).</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -2066,22 +2066,22 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>§1367(b) and (c): the exceptions</t>
+          <t>Rule 13(b): permissive counterclaim and Cordero v. Voltaire</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>(b): in a case resting only on diversity, no supplemental jx over claims by PLAINTIFFS against persons made parties under Rules 14, 19, 20 or 24 (or claims by would-be Rule 19/24 plaintiffs) when that would be inconsistent with §1332. (c): the court MAY decline supplemental jx, e.g., when the added claims would overwhelm the case.</t>
+          <t>PERMISSIVE counterclaim = UNRELATED to the plaintiff's claim. Rule 13 ALLOWS it, but supplemental jx won't work (it needs the same facts), so it must have an INDEPENDENT basis: federal question or diversity.</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>(b) applies only when the PLAINTIFF is adding the party in a diversity-only case. If the DEFENDANT adds a party (Rule 14), (b) doesn't block it. With a federal-question anchor, (b) doesn't apply at all.</t>
+          <t>Cordero v. Voltaire: no FQ, no diversity, so both counterclaims needed supplemental jx. Counterclaim I arose from the same nucleus of facts as the anchor → compulsory → stays. Counterclaim II came from a different nucleus of facts → permissive → DISMISSED from the federal suit. It isn't necessarily lost: it can be brought in STATE court.</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "§1367(b) bars a defendant's impleader of a non-diverse party." Wrong: applying (b) when the anchor is a federal question.</t>
+          <t>Wrong: "permissive counterclaims get supplemental jx." Wrong: "a dismissed permissive counterclaim is forfeited forever."</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -2098,22 +2098,22 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Rule 20: permissive joinder of parties</t>
+          <t>§1367(b) and (c): the exceptions</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Plaintiffs MAY join (20(a)(1)), and defendants MAY be joined (20(a)(2)), if BOTH: (A) a right to relief jointly, severally or in the alternative arising out of the SAME TRANSACTION, OCCURRENCE, or SERIES of them; AND (B) a QUESTION OF LAW OR FACT COMMON to all.</t>
+          <t>(b): in a case resting only on diversity, no supplemental jx over claims by PLAINTIFFS against persons made parties under Rules 14, 19, 20 or 24 (or claims by would-be Rule 19/24 plaintiffs) when that would be inconsistent with §1332. (c): the court MAY decline supplemental jx, e.g., when the added claims would overwhelm the case.</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Analyze every "arrow" (each P → each D): does Rule 20 allow it, and is there SMJ for it? Class example: P sues D for breach of contract; a friend wants to add an unrelated defamation claim → Rule 20 doesn't allow it (no common facts, no common legal question). Once Rule 20 fails, skip the SMJ analysis.</t>
+          <t>(b) applies only when the PLAINTIFF is adding the party in a diversity-only case. If the DEFENDANT adds a party (Rule 14), (b) doesn't block it. With a federal-question anchor, (b) doesn't apply at all.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>NOTES FIX: the Week 9 notes list the same-transaction + common-question preconditions under Rule 19. Those are Rule 20's elements. Rule 19 is REQUIRED joinder (complete relief / impaired interest / inconsistent obligations), raised by 12(b)(7). Wrong: "Rule 20 joinder is mandatory."</t>
+          <t>Wrong: "§1367(b) bars a defendant's impleader of a non-diverse party." Wrong: applying (b) when the anchor is a federal question.</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -2130,22 +2130,22 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Mosley v. General Motors (1974)</t>
+          <t>Rule 20: permissive joinder of parties</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Multiple plaintiffs (P1, P2, P3) each suing GM on their OWN federal discrimination claims may join under Rule 20 when their claims arise from the same SERIES of transactions or occurrences and share common questions of law and fact.</t>
+          <t>Plaintiffs MAY join (20(a)(1)), and defendants MAY be joined (20(a)(2)), if BOTH: (A) a right to relief jointly, severally or in the alternative arising out of the SAME TRANSACTION, OCCURRENCE, or SERIES of them; AND (B) a QUESTION OF LAW OR FACT COMMON to all.</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>GM's argument: the events were separate, a different nucleus of facts for each plaintiff. The court found common enough questions of fact and law to allow joinder. SMJ: each plaintiff has a federal claim → federal question for every arrow.</t>
+          <t>Analyze every "arrow" (each P → each D): does Rule 20 allow it, and is there SMJ for it? Class example: P sues D for breach of contract; a friend wants to add an unrelated defamation claim → Rule 20 doesn't allow it (no common facts, no common legal question). Once Rule 20 fails, skip the SMJ analysis.</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Wrong: "each plaintiff's injury must come from the exact same event." A series of related transactions can be enough.</t>
+          <t>NOTES FIX: the Week 9 notes list the same-transaction + common-question preconditions under Rule 19. Those are Rule 20's elements. Rule 19 is REQUIRED joinder (complete relief / impaired interest / inconsistent obligations), raised by 12(b)(7). Wrong: "Rule 20 joinder is mandatory."</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -2162,69 +2162,73 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
+          <t>Mosley v. General Motors (1974)</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Multiple plaintiffs (P1, P2, P3) each suing GM on their OWN federal discrimination claims may join under Rule 20 when their claims arise from the same SERIES of transactions or occurrences and share common questions of law and fact.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>GM's argument: the events were separate, a different nucleus of facts for each plaintiff. The court found common enough questions of fact and law to allow joinder. SMJ: each plaintiff has a federal claim → federal question for every arrow.</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Wrong: "each plaintiff's injury must come from the exact same event." A series of related transactions can be enough.</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Week 9 class notes (10/21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>12. JOINDER</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
           <t>Week 9 in-class hypos: Ann v. Barbara + Charles</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>(1) Ann (IL) sues Barbara (IL) under federal civil-rights law and joins co-worker Charles on a state tort claim (Rule 20 satisfied): YES, supplemental jx. The federal anchor supports §1367(a) jurisdiction over the related state claim, and §1367(b) doesn't apply because the anchor isn't diversity. (2) Ann (IL) sues Barbara (WI) for breach of contract (&gt; $75k, diversity only) and joins Charles (IL) for conspiracy (Rule 20 satisfied): NO. §1367(b) bars a plaintiff's claim against a party joined under Rule 20 when it would destroy complete diversity.</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>Same facts, same rule; the anchor decides it. Federal-question anchor → (b) doesn't apply. Diversity-only anchor + plaintiff adds a non-diverse defendant → (b) bars it.</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>Wrong: "supplemental jx works in both because the claims are related." Wrong: "no jx in #1 because Ann and Charles are both from Illinois" (citizenship doesn't matter with a federal anchor).</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>Week 9 class notes (10/21)</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>13. NOT YET COVERED</t>
         </is>
       </c>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>13. NOT YET COVERED</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>Erie (flag: not in Weeks 1-9)</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr"/>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Minimum contacts is a PJ test, not Erie.</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>20Q6, 20Q30</t>
-        </is>
-      </c>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2234,21 +2238,49 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Forum non conveniens (flag)</t>
+          <t>Erie (flag: not in Weeks 1-9)</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+          <t>Erie applies to a federal court with diversity jx (and to joined claims resting on diversity). Tests: purpose test; outcome-determinative test.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr"/>
       <c r="E64" s="5" t="inlineStr">
         <is>
+          <t>Minimum contacts is a PJ test, not Erie.</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>20Q6, 20Q30</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>13. NOT YET COVERED</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Forum non conveniens (flag)</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>A foreign defendant wanting a non-U.S. court moves to DISMISS for forum non conveniens.</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr"/>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
           <t>Not transfer (you can't transfer to a foreign court); not improper venue.</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
         <is>
           <t>20Q36</t>
         </is>
@@ -2266,7 +2298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2410,145 +2442,149 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Rule 22: interpleader</t>
+          <t>Rule 14: impleader (defendant adds a party)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A party facing DOUBLE OR MULTIPLE LIABILITY to competing claimants can bring them all into one action. (1) By a PLAINTIFF: join the claimants as defendants and require them to interplead. (2) By a DEFENDANT: through a crossclaim or counterclaim. Allowed even if the claims lack a common origin or are adverse and independent, and even if the stakeholder denies owing anyone. Rule 22 supplements Rule 20 and works alongside statutory interpleader (28 U.S.C. §§1335, 1397, 2361).</t>
+          <t>A defending party, as third-party plaintiff, may serve a summons and complaint on a nonparty 'who is or may be liable to it for all or part of the claim against it.' The defendant is PASSING ON liability: 'if I'm liable, this person must cover me in some way.' It needs an existing LEGAL obligation (indemnity, contract, insurance, contribution, warranty). It is NOT the defendant saying 'it wasn't me, it was him' (that's a defense). NEVER compulsory: the defendant can bring the claim against the third party in a later, separate suit.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>InsureCo holds a $100,000 life-insurance payout claimed by both the ex-wife and the current wife; it sues both and lets the court decide (plaintiff interpleader). Ana sues BankCo for her late father's account; BankCo brings in a creditor who also claims it (defendant interpleader). An escrow deposit claimed by a buyer and by a contractor under a separate assignment: no common origin, still OK.</t>
+          <t>Classic case: the defendant pulls in its own liability insurer. That is the defendant's claim against the insurer, not the plaintiff suing the insurer. Exam pattern: one fact pattern, with facts changed within it to ask whether and how the defendant can bring someone in.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Still needs SMJ (FQ or diversity) under Rule 22. Statutory interpleader: see the next row.</t>
+          <t>Defendant's claim against the third party: usually supplemental (same facts); §1367(b) does NOT bar it, because it limits only plaintiffs. Plaintiff's own claim against a non-diverse third-party defendant in a diversity-only case: barred (Kroger, §1367(b)).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Interpleader: the stakeholder's dilemma and Dunlevy (casebook p. 825)</t>
+          <t>Counterclaims by a third-party defendant</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>The problem: a husband's life insurance policy is payable to "my wife"; the couple divorces, he remarries and dies, and both wives claim the proceeds. If they bring separate suits, both may win. Same situation: two competing claimants each want to withdraw a small business's entire bank account. The stakeholder (insurer or bank) concedes it owes the money but wants a procedure that binds all claimants. Past difficulties: (1) no effective procedural device to join both claimants; (2) possible jurisdictional and venue limitations. INTERPLEADER lets a stakeholder (often a bank or insurer) require the competing claimants to litigate their rights to the fund or property. Rule 22 typifies such a joinder provision, and it allows interpleader even if the stakeholder asserts some claim on the assets itself (e.g., a bank reducing the account balance by an unpaid loan). Typically, the stakeholder invokes interpleader, joining the claimants as parties.</t>
+          <t>Once impleaded, the third-party defendant may counterclaim against the defendant (the third-party plaintiff) under Rule 13. Like any counterclaim, it may be related or unrelated: the RULE always allows it.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>New York Life Insurance Co. v. Dunlevy (1916): Father, in Pennsylvania, bought a policy paying a lump sum after a set number of years. When it came due, Father and Daughter disagreed over who was entitled. Daughter's creditor sued in Pennsylvania; the insurer interpleaded Father, Daughter and Creditor; the Pennsylvania court ruled for Father. Daughter sued the insurer in California. The Supreme Court held the Pennsylvania suit did NOT preclude her claim, because Pennsylvania had not acquired personal jurisdiction over Daughter, who lived in California. The insurer was liable a second time.</t>
+          <t>Insurer, impleaded by the defendant, counterclaims against the defendant for unpaid premiums (unrelated) or for a declaration of no coverage (related).</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>An interpleader proceeding fails to yield a stable resolution if the forum lacks jurisdiction over the claimants (Dunlevy).</t>
+          <t>Step 2 still applies: each counterclaim needs SMJ (federal question, diversity, or supplemental if related). An unrelated one needs its own basis.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Statutory interpleader (Federal Interpleader Act) vs. Rule 22 (casebook pp. 825-826)</t>
+          <t>Rule 22: interpleader</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Congress responded to Dunlevy-type problems with the Federal Interpleader Act, 28 U.S.C. §§1335, 1397, 2361. The Act: (1) broadens the circumstances in which interpleader is available, eliminating some restrictions older equity doctrines imposed (§1335); (2) removes limitations on federal SMJ (§1335(a)); (3) permits nationwide service of process, interpreted to mean nationwide personal jurisdiction (§2361); (4) expands venue to where any claimant resides (§1397). Rule 22 closely resembles the Act, BUT Rule 22 actions are subject to the NORMAL rules for SMJ (diversity between all plaintiffs and all defendants; amount in controversy), personal jurisdiction (jurisdiction within the state) and venue (residency of all defendants, or where the claim arises).</t>
+          <t>A party facing DOUBLE OR MULTIPLE LIABILITY to competing claimants can bring them all into one action. (1) By a PLAINTIFF: join the claimants as defendants and require them to interplead. (2) By a DEFENDANT: through a crossclaim or counterclaim. Allowed even if the claims lack a common origin or are adverse and independent, and even if the stakeholder denies owing anyone. Rule 22 supplements Rule 20 and works alongside statutory interpleader (28 U.S.C. §§1335, 1397, 2361).</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Dunlevy under the Act: Daughter would be subject to the jurisdiction of the federal courts in Pennsylvania (§2361), which could resolve all the parties' conflicting claims. In practice, Rule 22 is used when the stakeholder is a citizen of one state and all claimants are citizens of a second state: there is no jurisdiction under the Interpleader Act because no two claimants are diverse, but the normal rules for jurisdiction and venue can be satisfied by an action in the state of all claimants.</t>
+          <t>InsureCo holds a $100,000 life-insurance payout claimed by both the ex-wife and the current wife; it sues both and lets the court decide (plaintiff interpleader). Ana sues BankCo for her late father's account; BankCo brings in a creditor who also claims it (defendant interpleader). An escrow deposit claimed by a buyer and by a contractor under a separate assignment: no common origin, still OK.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Statutory: SMJ per §1335(a); nationwide PJ (§2361); venue where any claimant resides (§1397). Rule 22: normal SMJ (complete diversity + amount), normal PJ and normal venue.</t>
+          <t>Still needs SMJ (FQ or diversity) under Rule 22. Statutory interpleader: see the next row.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Rule 24: intervention</t>
+          <t>Interpleader: the stakeholder's dilemma and Dunlevy (casebook p. 825)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>A NON-PARTY asks to join. (a) AS OF RIGHT: the court MUST allow a TIMELY motion by anyone with (1) an unconditional statutory right, or (2) an interest in the property or transaction at issue that may be practically impaired, unless existing parties adequately represent it. (b) PERMISSIVE: the court MAY allow a TIMELY motion by anyone with (1) a conditional statutory right, or (2) a claim or defense sharing a common question of law or fact; (b)(2) government officers or agencies may intervene when the case involves a statute or order they administer; (b)(3) the court must consider undue delay or prejudice to the original parties. (c) PROCEDURE: a motion served under Rule 5, with a pleading stating the claim or defense.</t>
+          <t>The problem: a husband's life insurance policy is payable to "my wife"; the couple divorces, he remarries and dies, and both wives claim the proceeds. If they bring separate suits, both may win. Same situation: two competing claimants each want to withdraw a small business's entire bank account. The stakeholder (insurer or bank) concedes it owes the money but wants a procedure that binds all claimants. Past difficulties: (1) no effective procedural device to join both claimants; (2) possible jurisdictional and venue limitations. INTERPLEADER lets a stakeholder (often a bank or insurer) require the competing claimants to litigate their rights to the fund or property. Rule 22 typifies such a joinder provision, and it allows interpleader even if the stakeholder asserts some claim on the assets itself (e.g., a bank reducing the account balance by an unpaid loan). Typically, the stakeholder invokes interpleader, joining the claimants as parties.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>An environmental group protecting a wetland at issue: interest + possible impairment + inadequate representation → as of right, but only if timely (waiting 14 months until a week before trial fails). A business with a similar claim against the same defendant → permissive at most; the judge may say no.</t>
+          <t>New York Life Insurance Co. v. Dunlevy (1916): Father, in Pennsylvania, bought a policy paying a lump sum after a set number of years. When it came due, Father and Daughter disagreed over who was entitled. Daughter's creditor sued in Pennsylvania; the insurer interpleaded Father, Daughter and Creditor; the Pennsylvania court ruled for Father. Daughter sued the insurer in California. The Supreme Court held the Pennsylvania suit did NOT preclude her claim, because Pennsylvania had not acquired personal jurisdiction over Daughter, who lived in California. The insurer was liable a second time.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Every intervenor's claim still needs SMJ (FQ, diversity, or supplemental, subject to §1367(b) limits).</t>
+          <t>An interpleader proceeding fails to yield a stable resolution if the forum lacks jurisdiction over the claimants (Dunlevy).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Intervention: purpose, structure and the four Rule 24(a) requirements (casebook intro, through p. 813)</t>
+          <t>Statutory interpleader (Federal Interpleader Act) vs. Rule 22 (casebook pp. 825-826)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>PURPOSE: The other joinder devices bring in a party who does NOT want to be there; intervention does the opposite: it lets an unjoined person "elbow her way into a suit where no one wants her." Like compulsory joinder, it flows from the recognition that lawsuits may affect persons not joined. Those effects are not formal preclusion (due process forbids binding one who was not a party), but judgments have broader ripple effects than the decree's formal binding effect. COSTS: existing parties (and perhaps the judge) may be unenthusiastic; intervention complicates and perhaps weakens their strategy (even an intervenor seeking the same outcome has a different perspective and perhaps strategy), may make the suit more expensive and settlement harder, and erodes party autonomy; carried to a logical extreme it turns every lawsuit into a "town meeting." Intervention principles allow some, but not all, who wish to be involved to join. STRUCTURE: (1) INTERVENTION OF RIGHT, Rule 24(a): gives those with STRONG interests the power to insist on joinder; Rule 24(a)(2)'s words echo Rule 19(a)(1)(B) ("an interest relating to . . . the subject of the action . . . so situated that disposing of the action may as a practical matter impair or impede" the would-be intervenor's interests). An applicant who meets Rule 24(a) MUST be allowed to join. (2) PERMISSIVE INTERVENTION, Rule 24(b): the weaker counterpart, for those with weaker bases for insisting on joinder. An applicant who meets only Rule 24(b) MAY be allowed to join; the judge's decision is reviewed only for ABUSE OF DISCRETION. FOUR Rule 24(a) REQUIREMENTS (the focus of most reported cases): (1) TIMELY: the intervenor may not lie in wait until the litigation is on the brink of resolution; (2) an INTEREST in the property or transaction that is the subject of the suit; (3) that interest must be in some strong way AT RISK; (4) even an applicant meeting all of these is denied if those already in the suit ADEQUATELY REPRESENT the interest.</t>
+          <t>Congress responded to Dunlevy-type problems with the Federal Interpleader Act, 28 U.S.C. §§1335, 1397, 2361. The Act: (1) broadens the circumstances in which interpleader is available, eliminating some restrictions older equity doctrines imposed (§1335); (2) removes limitations on federal SMJ (§1335(a)); (3) permits nationwide service of process, interpreted to mean nationwide personal jurisdiction (§2361); (4) expands venue to where any claimant resides (§1397). Rule 22 closely resembles the Act, BUT Rule 22 actions are subject to the NORMAL rules for SMJ (diversity between all plaintiffs and all defendants; amount in controversy), personal jurisdiction (jurisdiction within the state) and venue (residency of all defendants, or where the claim arises).</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Developer and City Zoning Board litigate whether Developer can build an office building on a plot bordering a residential area. If Developer wins, Homeowner (next to the plot) is affected; if Developer loses, Landowner (owner of another adjacent plot that would be more valuable if commercially developed) is adversely affected. The judgment won't formally bind either, but will affect both, and both might wish to influence the outcome. If entitled to intervene, they would become parties with the right to present evidence and arguments like Developer and the Zoning Board. Next case: NRDC v. U.S. Nuclear Regulatory Commission (10th Cir. 1978): American Mining Congress and Kerr-McGee Nuclear Corp. sought review of the denial of their motions to intervene of right and permissively under Rule 24(a)(2) and (b); the casebook says the case assumes timeliness and analyzes the other three criteria.</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr"/>
+          <t>Dunlevy under the Act: Daughter would be subject to the jurisdiction of the federal courts in Pennsylvania (§2361), which could resolve all the parties' conflicting claims. In practice, Rule 22 is used when the stakeholder is a citizen of one state and all claimants are citizens of a second state: there is no jurisdiction under the Interpleader Act because no two claimants are diverse, but the normal rules for jurisdiction and venue can be satisfied by an action in the state of all claimants.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Statutory: SMJ per §1335(a); nationwide PJ (§2361); venue where any claimant resides (§1397). Rule 22: normal SMJ (complete diversity + amount), normal PJ and normal venue.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>§1367(b): the diversity exception</t>
+          <t>Rule 24: intervention</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+          <t>A NON-PARTY asks to join. (a) AS OF RIGHT: the court MUST allow a TIMELY motion by anyone with (1) an unconditional statutory right, or (2) an interest in the property or transaction at issue that may be practically impaired, unless existing parties adequately represent it. (b) PERMISSIVE: the court MAY allow a TIMELY motion by anyone with (1) a conditional statutory right, or (2) a claim or defense sharing a common question of law or fact; (b)(2) government officers or agencies may intervene when the case involves a statute or order they administer; (b)(3) the court must consider undue delay or prejudice to the original parties. (c) PROCEDURE: a motion served under Rule 5, with a pleading stating the claim or defense.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+          <t>An environmental group protecting a wetland at issue: interest + possible impairment + inadequate representation → as of right, but only if timely (waiting 14 months until a week before trial fails). A business with a similar claim against the same defendant → permissive at most; the judge may say no.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+          <t>Every intervenor's claim still needs SMJ (FQ, diversity, or supplemental, subject to §1367(b) limits).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>§1367(c): court may decline</t>
+          <t>Intervention: purpose, structure and the four Rule 24(a) requirements (casebook intro, through p. 813)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Even with supplemental jx, the court MAY decline it, e.g., when the added claims would overwhelm the case.</t>
+          <t>PURPOSE: The other joinder devices bring in a party who does NOT want to be there; intervention does the opposite: it lets an unjoined person "elbow her way into a suit where no one wants her." Like compulsory joinder, it flows from the recognition that lawsuits may affect persons not joined. Those effects are not formal preclusion (due process forbids binding one who was not a party), but judgments have broader ripple effects than the decree's formal binding effect. COSTS: existing parties (and perhaps the judge) may be unenthusiastic; intervention complicates and perhaps weakens their strategy (even an intervenor seeking the same outcome has a different perspective and perhaps strategy), may make the suit more expensive and settlement harder, and erodes party autonomy; carried to a logical extreme it turns every lawsuit into a "town meeting." Intervention principles allow some, but not all, who wish to be involved to join. STRUCTURE: (1) INTERVENTION OF RIGHT, Rule 24(a): gives those with STRONG interests the power to insist on joinder; Rule 24(a)(2)'s words echo Rule 19(a)(1)(B) ("an interest relating to . . . the subject of the action . . . so situated that disposing of the action may as a practical matter impair or impede" the would-be intervenor's interests). An applicant who meets Rule 24(a) MUST be allowed to join. (2) PERMISSIVE INTERVENTION, Rule 24(b): the weaker counterpart, for those with weaker bases for insisting on joinder. An applicant who meets only Rule 24(b) MAY be allowed to join; the judge's decision is reviewed only for ABUSE OF DISCRETION. FOUR Rule 24(a) REQUIREMENTS (the focus of most reported cases): (1) TIMELY: the intervenor may not lie in wait until the litigation is on the brink of resolution; (2) an INTEREST in the property or transaction that is the subject of the suit; (3) that interest must be in some strong way AT RISK; (4) even an applicant meeting all of these is denied if those already in the suit ADEQUATELY REPRESENT the interest.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Plaintiff piles many state claims onto one small federal claim.</t>
+          <t>Developer and City Zoning Board litigate whether Developer can build an office building on a plot bordering a residential area. If Developer wins, Homeowner (next to the plot) is affected; if Developer loses, Landowner (owner of another adjacent plot that would be more valuable if commercially developed) is adversely affected. The judgment won't formally bind either, but will affect both, and both might wish to influence the outcome. If entitled to intervene, they would become parties with the right to present evidence and arguments like Developer and the Zoning Board. Next case: NRDC v. U.S. Nuclear Regulatory Commission (10th Cir. 1978): American Mining Congress and Kerr-McGee Nuclear Corp. sought review of the denial of their motions to intervene of right and permissively under Rule 24(a)(2) and (b); the casebook says the case assumes timeliness and analyzes the other three criteria.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -2556,20 +2592,60 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>§1367(b): the diversity exception</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>In a DIVERSITY-ONLY case, a PLAINTIFF can't use supplemental jx for a claim against a party it added (e.g., under Rule 20) if that would break complete diversity. Doesn't apply when the DEFENDANT adds the party, or when the anchor is a federal question.</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Ann (IL) v. Barbara (IL), federal civil-rights claim; Ann adds Charles on a state claim → YES, supplemental. Ann (IL) v. Barbara (WI), contract (diversity only); Ann adds Charles (IL) → NO, (b) bars it.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>The anchor decides it: federal → (b) doesn't apply; diversity-only → (b) can bar it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>§1367(c): court may decline</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Even with supplemental jx, the court MAY decline it, e.g., when the claim raises a NOVEL or complex issue of state law, or when the added claims would OVERWHELM (substantially predominate over) the case. Only matters when the claim rests on supplemental jx; a claim with its own federal question or diversity basis isn't subject to (c). Rule 42 (separate trials) is an alternative way to keep a case manageable.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Plaintiff piles many state claims onto one small federal claim. A party who doesn't want to be joined argues: (1) no SMJ (no federal question, no diversity, not related enough for §1367(a)), and (2) even if supplemental jx exists, the court should decline it under §1367(c).</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Rule 42: court separates or consolidates</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Even if the joinder rule is met AND there's SMJ, the judge can still separate claims or consolidate cases. The judge is never obligated to let joinder happen.</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Six properly joined claims are confusing a jury → judge orders separate trials.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2796,7 +2872,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -2826,7 +2902,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -2856,7 +2932,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -2976,7 +3052,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -3006,7 +3082,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -3036,7 +3112,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -3066,7 +3142,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>43, 45</t>
+          <t>44, 46</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -3096,7 +3172,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -3246,7 +3322,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -3276,7 +3352,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>49, 45</t>
+          <t>50, 46</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -3306,7 +3382,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>49, 45</t>
+          <t>50, 46</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -3366,7 +3442,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -3396,7 +3472,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>36, 34, 32</t>
+          <t>37, 35, 33</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -3516,7 +3592,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -3546,7 +3622,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -3726,7 +3802,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -3756,7 +3832,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -3846,7 +3922,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>49, 45</t>
+          <t>50, 46</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -3876,7 +3952,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -3996,7 +4072,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -4086,7 +4162,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -4146,7 +4222,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>64</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -4206,7 +4282,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -4266,7 +4342,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -4296,7 +4372,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -4446,7 +4522,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>15, 45</t>
+          <t>15, 46</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -4536,7 +4612,7 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -4566,7 +4642,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -4596,7 +4672,7 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -4626,7 +4702,7 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
@@ -4686,7 +4762,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -4716,7 +4792,7 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -4746,7 +4822,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -4776,7 +4852,7 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -4866,7 +4942,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>64</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -4896,7 +4972,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -4926,7 +5002,7 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>21, 35</t>
+          <t>21, 36</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -5046,7 +5122,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>65</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
@@ -5166,7 +5242,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -5526,7 +5602,7 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>21, 31</t>
+          <t>21, 32</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -5586,7 +5662,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
@@ -5616,7 +5692,7 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -5646,7 +5722,7 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>23, 43</t>
+          <t>23, 44</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
@@ -5676,7 +5752,7 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>15, 45</t>
+          <t>15, 46</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -5766,7 +5842,7 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">

</xml_diff>